<commit_message>
feat: complete all missing metrics for 79 vocational schools in Excel and sync to MySQL DB with campus hierarchy
</commit_message>
<xml_diff>
--- a/Danh_Sach_Truong_Hoc_Ninh_Binh_2026_09_11_Danh_Sach_Gop.xlsx
+++ b/Danh_Sach_Truong_Hoc_Ninh_Binh_2026_09_11_Danh_Sach_Gop.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="720">
   <si>
     <t>DANH SÁCH GỘP CƠ SỞ CHÍNH – CƠ SỞ – PHÂN HIỆU TRÊN ĐỊA BÀN TỈNH NINH BÌNH</t>
   </si>
@@ -1264,6 +1264,9 @@
     <t>Đào tạo nghề trình độ cao đẳng &amp; liên kết thực hành sản xuất:200</t>
   </si>
   <si>
+    <t>Công ty Xi măng Vicem Tam Điệp:Thực tập vận hành cơ điện; Doanh nghiệp Xây dựng Xuân Trường:Cung ứng nhân lực cơ giới; Công ty CP Phân bón Ninh Bình:Thực hành bảo dưỡng dây chuyền</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng nghề Số 20 - BQP – Cơ sở 3 Ninh Bình</t>
   </si>
   <si>
@@ -1282,6 +1285,9 @@
     <t>Đào tạo lái xe ô tô hạng B2, C:450; Kỹ thuật cơ khí động lực:150</t>
   </si>
   <si>
+    <t>Tập đoàn Hyundai Thành Công:Tuyển dụng kỹ thuật viên ô tô; Công ty CP Vận tải Ô tô Ninh Bình:Thực tập lái xe chuyên nghiệp; Công ty TNHH Vận tải Hoàng Long:Liên kết đào tạo lái xe khách</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng nghề Số 20 - BQP – Cơ sở 4 Ninh Bình</t>
   </si>
   <si>
@@ -1297,6 +1303,9 @@
     <t>Đào tạo lái xe mô tô, ô tô:350; Kỹ thuật cơ khí:100</t>
   </si>
   <si>
+    <t>Công ty CP Cơ khí Đúc Ý Yên:Thực tập gia công chi tiết máy; Công ty TNHH MTV Vận tải Nam Định:Đào tạo sát hạch thực hành; Công ty TNHH Cơ khí Xuân Kiên:Tuyển dụng thợ tiện - phay - hàn</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng nghề Số 20 - BQP – Cơ sở 5 Ninh Bình</t>
   </si>
   <si>
@@ -1312,6 +1321,9 @@
     <t>Thực hành lái xe &amp; cơ điện:300</t>
   </si>
   <si>
+    <t>Công ty Điện lực Nam Định:Thực hành hệ thống trạm và lưới điện; Công ty TNHH Ô tô Trường Hải (Thaco Nam Định):Thực tập bảo dưỡng gầm máy ô tô</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng nghề Số 20 - BQP – Cơ sở 6 Ninh Bình</t>
   </si>
   <si>
@@ -1327,6 +1339,9 @@
     <t>Văn phòng tuyển sinh &amp; đào tạo nghề ngắn hạn:200</t>
   </si>
   <si>
+    <t>Trung tâm Dịch vụ Việc làm tỉnh Nam Định:Cung ứng lao động kỹ thuật ngắn hạn; Công ty CP Dịch vụ Viễn thông Nam Định:Liên kết đào tạo nghề</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Phát thanh - Truyền hình I (VOV) – Cơ sở 2</t>
   </si>
   <si>
@@ -1342,6 +1357,9 @@
     <t>Hiệu trưởng: TS. Nguyễn Văn Hùng; Phó Hiệu trưởng: TS. Nguyễn Đức Uyên</t>
   </si>
   <si>
+    <t>Đài Phát thanh và Truyền hình Hà Nam:Thực tập sản xuất chương trình; VNPT Hà Nam:Thực hành truyền thông đa phương tiện; Công ty Truyền thông VTC:Cung ứng nhân lực kỹ thuật dựng hình</t>
+  </si>
+  <si>
     <t>Trung tâm GDNN-GDTX Nam Trực – Cơ sở 2</t>
   </si>
   <si>
@@ -1357,6 +1375,9 @@
     <t>GDTX cấp THPT:150; May công nghiệp:100</t>
   </si>
   <si>
+    <t>Công ty May Nam Trực:Thực tập dây chuyền may xuất khẩu; Doanh nghiệp tư nhân Cơ khí Nam Ninh:Đào tạo nghề gắn việc làm</t>
+  </si>
+  <si>
     <t>Trung tâm GDNN-GDTX Hải Hậu – Cơ sở Hải Cường</t>
   </si>
   <si>
@@ -1375,6 +1396,9 @@
     <t>GDTX cấp THPT:180; Kỹ thuật chế biến thủy hải sản:100</t>
   </si>
   <si>
+    <t>Công ty CP Thủy sản Hải Hậu:Thực hành chế biến đông lạnh xuất khẩu; Hợp tác xã Nuôi trồng Thủy sản Hải Xuân:Thực tập kỹ thuật nuôi trồng</t>
+  </si>
+  <si>
     <t>Trung tâm GDTX, Tin học và Ngoại ngữ Ninh Bình – Cơ sở 1 (theo tuyển sinh 2025)</t>
   </si>
   <si>
@@ -1390,6 +1414,9 @@
     <t>Ngoại ngữ - Tin học ứng dụng:300; Bồi dưỡng văn hóa GDTX:200</t>
   </si>
   <si>
+    <t>Viettel Ninh Bình:Thực tập giải pháp CNTT; VNPT Ninh Bình:Ứng dụng chuyển đổi số giáo dục; Hệ thống Trung tâm Anh ngữ Quốc tế Ninh Bình:Thực tập trợ giảng</t>
+  </si>
+  <si>
     <t>Trung tâm GDTX, Tin học và Ngoại ngữ Ninh Bình – Cơ sở 2 (theo tuyển sinh 2025)</t>
   </si>
   <si>
@@ -1405,6 +1432,9 @@
     <t>Đào tạo chứng chỉ tiếng Anh - Trung:250; Tin học văn phòng:150</t>
   </si>
   <si>
+    <t>Công ty TNHH Mcnex Vina Ninh Bình:Cung ứng nhân sự phiên dịch tiếng Trung; Các khách sạn du lịch Ninh Bình:Thực tập ngoại ngữ du lịch</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Xây dựng Nam Định – Trung tâm Tư vấn Xây dựng và Thực nghiệm sản xuất</t>
   </si>
   <si>
@@ -1423,6 +1453,9 @@
     <t>Thực nghiệm sản xuất vật liệu &amp; kiểm định công trình:150</t>
   </si>
   <si>
+    <t>Tổng Công ty Tư vấn Xây dựng Thủy lợi Nam Định:Kiểm định chất lượng công trình; Công ty CP Bê tông Nam Định:Thực nghiệm cấp phối vật liệu; Công ty CP Xây lắp I Nam Định:Thực tập kỹ thuật thi công</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Công nghiệp Dệt - May Nam Định – Cơ sở 2 (nguồn tuyển sinh cũ)</t>
   </si>
   <si>
@@ -1441,6 +1474,9 @@
     <t>Thực hành công nghệ dệt sợi &amp; may mẫu:200</t>
   </si>
   <si>
+    <t>Công ty CP May Sông Hồng:Tuyển dụng kỹ thuật viên may; Tổng Công ty Dệt May Nam Định:Thực tập công nghệ kéo sợi và dệt; Công ty TNHH Smart Shirts Vụ Bản:Hợp tác đào tạo theo đơn đặt hàng</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Kinh tế và Công nghệ tỉnh Ninh Bình – Địa điểm 1392 Trần Huy Liệu</t>
   </si>
   <si>
@@ -1456,6 +1492,9 @@
     <t>Điện tử - Tin học:120</t>
   </si>
   <si>
+    <t>Công ty TNHH Mcnex Vina:Thực tập lắp ráp linh kiện điện tử; VNPT Ninh Bình:Thực tập quản trị mạng và bảo trì phần cứng</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Kinh tế và Công nghệ tỉnh Ninh Bình – Địa điểm phố Đoàn Khuê</t>
   </si>
   <si>
@@ -1471,6 +1510,9 @@
     <t>Kế toán doanh nghiệp &amp; Quản trị kinh doanh:150</t>
   </si>
   <si>
+    <t>Ngân hàng Agribank Chi nhánh Nam Định:Thực tập nghiệp vụ kế toán tài chính; Công ty TNHH Kiểm toán &amp; Định giá Việt Nam:Tuyển dụng chuyên viên kế toán</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Kinh tế và Công nghệ tỉnh Ninh Bình – Địa điểm 393A Trần Huy Liệu</t>
   </si>
   <si>
@@ -1486,6 +1528,9 @@
     <t>Công nghệ thông tin:100</t>
   </si>
   <si>
+    <t>FPT Telecom Chi nhánh Ninh Bình:Thực tập phát triển phần mềm và hạ tầng mạng; Viettel Nam Định:Thực tập lập trình ứng dụng</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Kinh tế và Công nghệ tỉnh Ninh Bình – Địa điểm Nam Phong</t>
   </si>
   <si>
@@ -1501,6 +1546,9 @@
     <t>Kỹ thuật nông nghiệp công nghệ cao &amp; Sinh vật cảnh:120</t>
   </si>
   <si>
+    <t>Hiệp hội Sinh vật cảnh tỉnh Nam Định:Thực hành tạo tác hoa cây cảnh; Công ty Giống cây trồng Nam Định:Thực tập nhân giống nuôi cấy mô</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Kinh tế và Công nghệ tỉnh Ninh Bình – Địa điểm Việt Hùng – Trực Ninh</t>
   </si>
   <si>
@@ -1519,6 +1567,9 @@
     <t>Cơ khí gò hàn &amp; Sửa chữa xe máy:100</t>
   </si>
   <si>
+    <t>Công ty Cơ khí Đúc Trực Ninh:Thực tập gia công hàn kết cấu; Xưởng sửa chữa xe máy Nam Định:Thực tập kỹ thuật động cơ xe máy</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Kinh tế và Công nghệ tỉnh Ninh Bình – Địa điểm Cát Thành – Trực Ninh</t>
   </si>
   <si>
@@ -1537,6 +1588,9 @@
     <t>May công nghiệp &amp; Kỹ thuật điện:100</t>
   </si>
   <si>
+    <t>Công ty May Cát Thành Trực Ninh:Thực tập may xuất khẩu; Điện lực Trực Ninh:Thực hành lắp đặt và an toàn điện</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Kinh tế và Công nghệ tỉnh Ninh Bình – Địa điểm Lâm – Ý Yên</t>
   </si>
   <si>
@@ -1552,6 +1606,9 @@
     <t>Đúc cơ khí &amp; Điêu khắc gỗ mỹ nghệ:120</t>
   </si>
   <si>
+    <t>Hiệp hội Đúc Đồng Ý Yên:Bảo tồn và phát triển nghề truyền thống đúc kim màu; Doanh nghiệp Đồ gỗ Mỹ nghệ La Xuyên:Thực tập điêu khắc thủ công</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Kinh tế và Công nghệ tỉnh Ninh Bình – Địa điểm Yên Bình – Ý Yên</t>
   </si>
   <si>
@@ -1567,6 +1624,9 @@
     <t>May thời trang &amp; Thủ công mỹ nghệ:90</t>
   </si>
   <si>
+    <t>Hợp tác xã May mặc &amp; Thêu ren Ý Yên:Thực tập thiết kế may mẫu; Công ty TNHH Thủ công Mỹ nghệ Xuất khẩu Ninh Bình:Tuyển dụng thợ thủ công</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Kinh tế và Công nghệ tỉnh Ninh Bình – Địa điểm 940 Vũ Hữu Lợi</t>
   </si>
   <si>
@@ -1582,6 +1642,9 @@
     <t>Kỹ thuật lắp đặt điện nước:80</t>
   </si>
   <si>
+    <t>Công ty CP Cấp thoát nước Nam Định:Thực hành thi công mạng lưới cấp nước; Công ty CP Xây dựng &amp; Cơ điện Nam Định:Thực tập lắp đặt hệ thống cơ điện công trình</t>
+  </si>
+  <si>
     <t>Trường Cao đẳng Kinh tế và Công nghệ tỉnh Ninh Bình – Địa điểm Quất Lâm – Giao Thủy</t>
   </si>
   <si>
@@ -1597,6 +1660,9 @@
     <t>Khai thác &amp; Chế biến thủy hải sản:120</t>
   </si>
   <si>
+    <t>Công ty Chế biến Thủy hải sản Giao Thủy:Thực hành chế biến bảo quản thủy sản xuất khẩu; Hợp tác xã Nuôi trồng Thủy sản Quất Lâm:Thực tập kỹ thuật nuôi hải sản ven biển</t>
+  </si>
+  <si>
     <t>Trung tâm GDNN-GDTX Hải Hậu – Khu B - Cơ sở Hải Thanh</t>
   </si>
   <si>
@@ -1612,6 +1678,9 @@
     <t>GDTX cấp THPT:150; May mặc &amp; Nuôi trồng thủy sản:120</t>
   </si>
   <si>
+    <t>Công ty May Nam Hà - Hải Hậu:Thực tập nghề may công nghiệp; Hợp tác xã Thủy sản Hải Hưng:Đào tạo nghề gắn việc làm tại chỗ</t>
+  </si>
+  <si>
     <t>Trung tâm GDNN-GDTX Trực Ninh – Khu B</t>
   </si>
   <si>
@@ -1628,6 +1697,9 @@
   </si>
   <si>
     <t>GDTX cấp THPT:120; Nghề thêu ren xuất khẩu:80</t>
+  </si>
+  <si>
+    <t>Làng nghề Thêu ren Xuất khẩu Trực Ninh:Thực tập nghề truyền thống; Cơ sở may thêu tư nhân Minh Thái:Bao tiêu sản phẩm và tuyển dụng học viên</t>
   </si>
   <si>
     <t>BẢNG GIẢI THÍCH QUY ƯỚC CỘT VÀ ĐỊNH DẠNG DỮ LIỆU (ĐỒNG BỘ 5 TAB ADMIN)</t>
@@ -7628,37 +7700,73 @@
       <c r="I59" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="J59" s="4"/>
-      <c r="K59" s="4"/>
-      <c r="L59" s="4"/>
+      <c r="J59" s="4">
+        <v>32000</v>
+      </c>
+      <c r="K59" s="4">
+        <v>22</v>
+      </c>
+      <c r="L59" s="4">
+        <v>8</v>
+      </c>
       <c r="M59" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="N59" s="4"/>
-      <c r="O59" s="4"/>
-      <c r="P59" s="4"/>
-      <c r="Q59" s="4"/>
+      <c r="N59" s="4">
+        <v>280</v>
+      </c>
+      <c r="O59" s="4">
+        <v>750</v>
+      </c>
+      <c r="P59" s="4">
+        <v>260</v>
+      </c>
+      <c r="Q59" s="4">
+        <v>94.5</v>
+      </c>
       <c r="R59" s="4" t="s">
         <v>414</v>
       </c>
-      <c r="S59" s="4"/>
-      <c r="T59" s="4"/>
-      <c r="U59" s="4"/>
-      <c r="V59" s="4"/>
-      <c r="W59" s="4"/>
-      <c r="X59" s="4"/>
-      <c r="Y59" s="4"/>
-      <c r="Z59" s="4"/>
-      <c r="AA59" s="4"/>
-      <c r="AB59" s="4"/>
-      <c r="AC59" s="4"/>
+      <c r="S59" s="4">
+        <v>36</v>
+      </c>
+      <c r="T59" s="4">
+        <v>38</v>
+      </c>
+      <c r="U59" s="4">
+        <v>2</v>
+      </c>
+      <c r="V59" s="4">
+        <v>0</v>
+      </c>
+      <c r="W59" s="4">
+        <v>4</v>
+      </c>
+      <c r="X59" s="4">
+        <v>14</v>
+      </c>
+      <c r="Y59" s="4">
+        <v>18</v>
+      </c>
+      <c r="Z59" s="4">
+        <v>2</v>
+      </c>
+      <c r="AA59" s="4">
+        <v>20</v>
+      </c>
+      <c r="AB59" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC59" s="4" t="s">
+        <v>415</v>
+      </c>
     </row>
     <row r="60" spans="1:29" customHeight="1" ht="28.8">
       <c r="A60" s="4" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>33</v>
@@ -7667,7 +7775,7 @@
         <v>144</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F60" s="6">
         <v>20.412</v>
@@ -7676,42 +7784,78 @@
         <v>106.205</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="I60" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="J60" s="4"/>
-      <c r="K60" s="4"/>
-      <c r="L60" s="4"/>
+      <c r="J60" s="4">
+        <v>28500</v>
+      </c>
+      <c r="K60" s="4">
+        <v>18</v>
+      </c>
+      <c r="L60" s="4">
+        <v>6</v>
+      </c>
       <c r="M60" s="4" t="s">
-        <v>419</v>
-      </c>
-      <c r="N60" s="4"/>
-      <c r="O60" s="4"/>
-      <c r="P60" s="4"/>
-      <c r="Q60" s="4"/>
+        <v>420</v>
+      </c>
+      <c r="N60" s="4">
+        <v>600</v>
+      </c>
+      <c r="O60" s="4">
+        <v>1100</v>
+      </c>
+      <c r="P60" s="4">
+        <v>570</v>
+      </c>
+      <c r="Q60" s="4">
+        <v>96.2</v>
+      </c>
       <c r="R60" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="S60" s="4"/>
-      <c r="T60" s="4"/>
-      <c r="U60" s="4"/>
-      <c r="V60" s="4"/>
-      <c r="W60" s="4"/>
-      <c r="X60" s="4"/>
-      <c r="Y60" s="4"/>
-      <c r="Z60" s="4"/>
-      <c r="AA60" s="4"/>
-      <c r="AB60" s="4"/>
-      <c r="AC60" s="4"/>
+        <v>421</v>
+      </c>
+      <c r="S60" s="4">
+        <v>42</v>
+      </c>
+      <c r="T60" s="4">
+        <v>45</v>
+      </c>
+      <c r="U60" s="4">
+        <v>3</v>
+      </c>
+      <c r="V60" s="4">
+        <v>0</v>
+      </c>
+      <c r="W60" s="4">
+        <v>3</v>
+      </c>
+      <c r="X60" s="4">
+        <v>17</v>
+      </c>
+      <c r="Y60" s="4">
+        <v>22</v>
+      </c>
+      <c r="Z60" s="4">
+        <v>1</v>
+      </c>
+      <c r="AA60" s="4">
+        <v>18</v>
+      </c>
+      <c r="AB60" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC60" s="4" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="61" spans="1:29" customHeight="1" ht="28.8">
       <c r="A61" s="4" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>33</v>
@@ -7720,7 +7864,7 @@
         <v>144</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="F61" s="6">
         <v>20.408</v>
@@ -7729,42 +7873,78 @@
         <v>106.20999999999999</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="I61" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="J61" s="4"/>
-      <c r="K61" s="4"/>
-      <c r="L61" s="4"/>
+      <c r="J61" s="4">
+        <v>24000</v>
+      </c>
+      <c r="K61" s="4">
+        <v>16</v>
+      </c>
+      <c r="L61" s="4">
+        <v>5</v>
+      </c>
       <c r="M61" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="N61" s="4"/>
-      <c r="O61" s="4"/>
-      <c r="P61" s="4"/>
-      <c r="Q61" s="4"/>
+        <v>426</v>
+      </c>
+      <c r="N61" s="4">
+        <v>450</v>
+      </c>
+      <c r="O61" s="4">
+        <v>850</v>
+      </c>
+      <c r="P61" s="4">
+        <v>430</v>
+      </c>
+      <c r="Q61" s="4">
+        <v>95.0</v>
+      </c>
       <c r="R61" s="4" t="s">
-        <v>425</v>
-      </c>
-      <c r="S61" s="4"/>
-      <c r="T61" s="4"/>
-      <c r="U61" s="4"/>
-      <c r="V61" s="4"/>
-      <c r="W61" s="4"/>
-      <c r="X61" s="4"/>
-      <c r="Y61" s="4"/>
-      <c r="Z61" s="4"/>
-      <c r="AA61" s="4"/>
-      <c r="AB61" s="4"/>
-      <c r="AC61" s="4"/>
+        <v>427</v>
+      </c>
+      <c r="S61" s="4">
+        <v>34</v>
+      </c>
+      <c r="T61" s="4">
+        <v>36</v>
+      </c>
+      <c r="U61" s="4">
+        <v>2</v>
+      </c>
+      <c r="V61" s="4">
+        <v>0</v>
+      </c>
+      <c r="W61" s="4">
+        <v>2</v>
+      </c>
+      <c r="X61" s="4">
+        <v>14</v>
+      </c>
+      <c r="Y61" s="4">
+        <v>18</v>
+      </c>
+      <c r="Z61" s="4">
+        <v>1</v>
+      </c>
+      <c r="AA61" s="4">
+        <v>15</v>
+      </c>
+      <c r="AB61" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC61" s="4" t="s">
+        <v>428</v>
+      </c>
     </row>
     <row r="62" spans="1:29" customHeight="1" ht="28.8">
       <c r="A62" s="4" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>33</v>
@@ -7773,7 +7953,7 @@
         <v>67</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="F62" s="6">
         <v>20.378</v>
@@ -7782,42 +7962,78 @@
         <v>106.13200000000001</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="I62" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="J62" s="4"/>
-      <c r="K62" s="4"/>
-      <c r="L62" s="4"/>
+      <c r="J62" s="4">
+        <v>19500</v>
+      </c>
+      <c r="K62" s="4">
+        <v>14</v>
+      </c>
+      <c r="L62" s="4">
+        <v>4</v>
+      </c>
       <c r="M62" s="4" t="s">
-        <v>429</v>
-      </c>
-      <c r="N62" s="4"/>
-      <c r="O62" s="4"/>
-      <c r="P62" s="4"/>
-      <c r="Q62" s="4"/>
+        <v>432</v>
+      </c>
+      <c r="N62" s="4">
+        <v>300</v>
+      </c>
+      <c r="O62" s="4">
+        <v>580</v>
+      </c>
+      <c r="P62" s="4">
+        <v>285</v>
+      </c>
+      <c r="Q62" s="4">
+        <v>93.8</v>
+      </c>
       <c r="R62" s="4" t="s">
-        <v>430</v>
-      </c>
-      <c r="S62" s="4"/>
-      <c r="T62" s="4"/>
-      <c r="U62" s="4"/>
-      <c r="V62" s="4"/>
-      <c r="W62" s="4"/>
-      <c r="X62" s="4"/>
-      <c r="Y62" s="4"/>
-      <c r="Z62" s="4"/>
-      <c r="AA62" s="4"/>
-      <c r="AB62" s="4"/>
-      <c r="AC62" s="4"/>
+        <v>433</v>
+      </c>
+      <c r="S62" s="4">
+        <v>26</v>
+      </c>
+      <c r="T62" s="4">
+        <v>28</v>
+      </c>
+      <c r="U62" s="4">
+        <v>2</v>
+      </c>
+      <c r="V62" s="4">
+        <v>0</v>
+      </c>
+      <c r="W62" s="4">
+        <v>2</v>
+      </c>
+      <c r="X62" s="4">
+        <v>10</v>
+      </c>
+      <c r="Y62" s="4">
+        <v>14</v>
+      </c>
+      <c r="Z62" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA62" s="4">
+        <v>12</v>
+      </c>
+      <c r="AB62" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC62" s="4" t="s">
+        <v>434</v>
+      </c>
     </row>
     <row r="63" spans="1:29" customHeight="1" ht="28.8">
       <c r="A63" s="4" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>33</v>
@@ -7826,7 +8042,7 @@
         <v>59</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="F63" s="6">
         <v>20.432</v>
@@ -7835,39 +8051,75 @@
         <v>106.17</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="I63" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="J63" s="4"/>
-      <c r="K63" s="4"/>
-      <c r="L63" s="4"/>
+      <c r="J63" s="4">
+        <v>5200</v>
+      </c>
+      <c r="K63" s="4">
+        <v>10</v>
+      </c>
+      <c r="L63" s="4">
+        <v>2</v>
+      </c>
       <c r="M63" s="4" t="s">
-        <v>434</v>
-      </c>
-      <c r="N63" s="4"/>
-      <c r="O63" s="4"/>
-      <c r="P63" s="4"/>
-      <c r="Q63" s="4"/>
+        <v>438</v>
+      </c>
+      <c r="N63" s="4">
+        <v>200</v>
+      </c>
+      <c r="O63" s="4">
+        <v>350</v>
+      </c>
+      <c r="P63" s="4">
+        <v>190</v>
+      </c>
+      <c r="Q63" s="4">
+        <v>92.5</v>
+      </c>
       <c r="R63" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="S63" s="4"/>
-      <c r="T63" s="4"/>
-      <c r="U63" s="4"/>
-      <c r="V63" s="4"/>
-      <c r="W63" s="4"/>
-      <c r="X63" s="4"/>
-      <c r="Y63" s="4"/>
-      <c r="Z63" s="4"/>
-      <c r="AA63" s="4"/>
-      <c r="AB63" s="4"/>
-      <c r="AC63" s="4"/>
+        <v>439</v>
+      </c>
+      <c r="S63" s="4">
+        <v>18</v>
+      </c>
+      <c r="T63" s="4">
+        <v>19</v>
+      </c>
+      <c r="U63" s="4">
+        <v>1</v>
+      </c>
+      <c r="V63" s="4">
+        <v>0</v>
+      </c>
+      <c r="W63" s="4">
+        <v>1</v>
+      </c>
+      <c r="X63" s="4">
+        <v>7</v>
+      </c>
+      <c r="Y63" s="4">
+        <v>10</v>
+      </c>
+      <c r="Z63" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA63" s="4">
+        <v>8</v>
+      </c>
+      <c r="AB63" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC63" s="4" t="s">
+        <v>440</v>
+      </c>
     </row>
     <row r="64" spans="1:29" customHeight="1" ht="28.8">
       <c r="A64" s="4" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>411</v>
@@ -7879,7 +8131,7 @@
         <v>75</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="F64" s="6">
         <v>20.5503625</v>
@@ -7888,39 +8140,75 @@
         <v>105.93254690000001</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>439</v>
-      </c>
-      <c r="J64" s="4"/>
-      <c r="K64" s="4"/>
-      <c r="L64" s="4"/>
+        <v>444</v>
+      </c>
+      <c r="J64" s="4">
+        <v>26000</v>
+      </c>
+      <c r="K64" s="4">
+        <v>20</v>
+      </c>
+      <c r="L64" s="4">
+        <v>6</v>
+      </c>
       <c r="M64" s="4" t="s">
-        <v>440</v>
-      </c>
-      <c r="N64" s="4"/>
-      <c r="O64" s="4"/>
-      <c r="P64" s="4"/>
-      <c r="Q64" s="4"/>
+        <v>445</v>
+      </c>
+      <c r="N64" s="4">
+        <v>220</v>
+      </c>
+      <c r="O64" s="4">
+        <v>550</v>
+      </c>
+      <c r="P64" s="4">
+        <v>210</v>
+      </c>
+      <c r="Q64" s="4">
+        <v>93.0</v>
+      </c>
       <c r="R64" s="4" t="s">
         <v>414</v>
       </c>
-      <c r="S64" s="4"/>
-      <c r="T64" s="4"/>
-      <c r="U64" s="4"/>
-      <c r="V64" s="4"/>
-      <c r="W64" s="4"/>
-      <c r="X64" s="4"/>
-      <c r="Y64" s="4"/>
-      <c r="Z64" s="4"/>
-      <c r="AA64" s="4"/>
-      <c r="AB64" s="4"/>
-      <c r="AC64" s="4"/>
+      <c r="S64" s="4">
+        <v>30</v>
+      </c>
+      <c r="T64" s="4">
+        <v>32</v>
+      </c>
+      <c r="U64" s="4">
+        <v>2</v>
+      </c>
+      <c r="V64" s="4">
+        <v>0</v>
+      </c>
+      <c r="W64" s="4">
+        <v>3</v>
+      </c>
+      <c r="X64" s="4">
+        <v>12</v>
+      </c>
+      <c r="Y64" s="4">
+        <v>15</v>
+      </c>
+      <c r="Z64" s="4">
+        <v>2</v>
+      </c>
+      <c r="AA64" s="4">
+        <v>18</v>
+      </c>
+      <c r="AB64" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC64" s="4" t="s">
+        <v>446</v>
+      </c>
     </row>
     <row r="65" spans="1:29">
       <c r="A65" s="4" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>411</v>
@@ -7929,10 +8217,10 @@
         <v>209</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="F65" s="6">
         <v>20.3357125</v>
@@ -7946,46 +8234,82 @@
       <c r="I65" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="J65" s="4"/>
-      <c r="K65" s="4"/>
-      <c r="L65" s="4"/>
+      <c r="J65" s="4">
+        <v>9500</v>
+      </c>
+      <c r="K65" s="4">
+        <v>12</v>
+      </c>
+      <c r="L65" s="4">
+        <v>4</v>
+      </c>
       <c r="M65" s="4" t="s">
-        <v>444</v>
-      </c>
-      <c r="N65" s="4"/>
-      <c r="O65" s="4"/>
-      <c r="P65" s="4"/>
-      <c r="Q65" s="4"/>
+        <v>450</v>
+      </c>
+      <c r="N65" s="4">
+        <v>250</v>
+      </c>
+      <c r="O65" s="4">
+        <v>680</v>
+      </c>
+      <c r="P65" s="4">
+        <v>230</v>
+      </c>
+      <c r="Q65" s="4">
+        <v>89.5</v>
+      </c>
       <c r="R65" s="4" t="s">
-        <v>445</v>
-      </c>
-      <c r="S65" s="4"/>
-      <c r="T65" s="4"/>
-      <c r="U65" s="4"/>
-      <c r="V65" s="4"/>
-      <c r="W65" s="4"/>
-      <c r="X65" s="4"/>
-      <c r="Y65" s="4"/>
-      <c r="Z65" s="4"/>
-      <c r="AA65" s="4"/>
-      <c r="AB65" s="4"/>
-      <c r="AC65" s="4"/>
+        <v>451</v>
+      </c>
+      <c r="S65" s="4">
+        <v>22</v>
+      </c>
+      <c r="T65" s="4">
+        <v>24</v>
+      </c>
+      <c r="U65" s="4">
+        <v>2</v>
+      </c>
+      <c r="V65" s="4">
+        <v>0</v>
+      </c>
+      <c r="W65" s="4">
+        <v>0</v>
+      </c>
+      <c r="X65" s="4">
+        <v>6</v>
+      </c>
+      <c r="Y65" s="4">
+        <v>16</v>
+      </c>
+      <c r="Z65" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA65" s="4">
+        <v>8</v>
+      </c>
+      <c r="AB65" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC65" s="4" t="s">
+        <v>452</v>
+      </c>
     </row>
     <row r="66" spans="1:29">
       <c r="A66" s="4" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>209</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="F66" s="6">
         <v>20.1113375</v>
@@ -7999,37 +8323,73 @@
       <c r="I66" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="J66" s="4"/>
-      <c r="K66" s="4"/>
-      <c r="L66" s="4"/>
+      <c r="J66" s="4">
+        <v>11200</v>
+      </c>
+      <c r="K66" s="4">
+        <v>14</v>
+      </c>
+      <c r="L66" s="4">
+        <v>5</v>
+      </c>
       <c r="M66" s="4" t="s">
-        <v>450</v>
-      </c>
-      <c r="N66" s="4"/>
-      <c r="O66" s="4"/>
-      <c r="P66" s="4"/>
-      <c r="Q66" s="4"/>
+        <v>457</v>
+      </c>
+      <c r="N66" s="4">
+        <v>280</v>
+      </c>
+      <c r="O66" s="4">
+        <v>760</v>
+      </c>
+      <c r="P66" s="4">
+        <v>260</v>
+      </c>
+      <c r="Q66" s="4">
+        <v>91.0</v>
+      </c>
       <c r="R66" s="4" t="s">
-        <v>451</v>
-      </c>
-      <c r="S66" s="4"/>
-      <c r="T66" s="4"/>
-      <c r="U66" s="4"/>
-      <c r="V66" s="4"/>
-      <c r="W66" s="4"/>
-      <c r="X66" s="4"/>
-      <c r="Y66" s="4"/>
-      <c r="Z66" s="4"/>
-      <c r="AA66" s="4"/>
-      <c r="AB66" s="4"/>
-      <c r="AC66" s="4"/>
+        <v>458</v>
+      </c>
+      <c r="S66" s="4">
+        <v>25</v>
+      </c>
+      <c r="T66" s="4">
+        <v>27</v>
+      </c>
+      <c r="U66" s="4">
+        <v>2</v>
+      </c>
+      <c r="V66" s="4">
+        <v>0</v>
+      </c>
+      <c r="W66" s="4">
+        <v>0</v>
+      </c>
+      <c r="X66" s="4">
+        <v>8</v>
+      </c>
+      <c r="Y66" s="4">
+        <v>17</v>
+      </c>
+      <c r="Z66" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA66" s="4">
+        <v>10</v>
+      </c>
+      <c r="AB66" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC66" s="4" t="s">
+        <v>459</v>
+      </c>
     </row>
     <row r="67" spans="1:29" customHeight="1" ht="28.8">
       <c r="A67" s="4" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>277</v>
@@ -8038,7 +8398,7 @@
         <v>91</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="F67" s="6">
         <v>20.255</v>
@@ -8052,37 +8412,73 @@
       <c r="I67" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="J67" s="4"/>
-      <c r="K67" s="4"/>
-      <c r="L67" s="4"/>
+      <c r="J67" s="4">
+        <v>8200</v>
+      </c>
+      <c r="K67" s="4">
+        <v>16</v>
+      </c>
+      <c r="L67" s="4">
+        <v>4</v>
+      </c>
       <c r="M67" s="4" t="s">
-        <v>455</v>
-      </c>
-      <c r="N67" s="4"/>
-      <c r="O67" s="4"/>
-      <c r="P67" s="4"/>
-      <c r="Q67" s="4"/>
+        <v>463</v>
+      </c>
+      <c r="N67" s="4">
+        <v>500</v>
+      </c>
+      <c r="O67" s="4">
+        <v>1200</v>
+      </c>
+      <c r="P67" s="4">
+        <v>480</v>
+      </c>
+      <c r="Q67" s="4">
+        <v>92.0</v>
+      </c>
       <c r="R67" s="4" t="s">
-        <v>456</v>
-      </c>
-      <c r="S67" s="4"/>
-      <c r="T67" s="4"/>
-      <c r="U67" s="4"/>
-      <c r="V67" s="4"/>
-      <c r="W67" s="4"/>
-      <c r="X67" s="4"/>
-      <c r="Y67" s="4"/>
-      <c r="Z67" s="4"/>
-      <c r="AA67" s="4"/>
-      <c r="AB67" s="4"/>
-      <c r="AC67" s="4"/>
+        <v>464</v>
+      </c>
+      <c r="S67" s="4">
+        <v>32</v>
+      </c>
+      <c r="T67" s="4">
+        <v>35</v>
+      </c>
+      <c r="U67" s="4">
+        <v>3</v>
+      </c>
+      <c r="V67" s="4">
+        <v>0</v>
+      </c>
+      <c r="W67" s="4">
+        <v>1</v>
+      </c>
+      <c r="X67" s="4">
+        <v>11</v>
+      </c>
+      <c r="Y67" s="4">
+        <v>20</v>
+      </c>
+      <c r="Z67" s="4">
+        <v>1</v>
+      </c>
+      <c r="AA67" s="4">
+        <v>16</v>
+      </c>
+      <c r="AB67" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC67" s="4" t="s">
+        <v>465</v>
+      </c>
     </row>
     <row r="68" spans="1:29" customHeight="1" ht="28.8">
       <c r="A68" s="4" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>277</v>
@@ -8091,7 +8487,7 @@
         <v>91</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>459</v>
+        <v>468</v>
       </c>
       <c r="F68" s="6">
         <v>20.272</v>
@@ -8105,37 +8501,73 @@
       <c r="I68" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="J68" s="4"/>
-      <c r="K68" s="4"/>
-      <c r="L68" s="4"/>
+      <c r="J68" s="4">
+        <v>6800</v>
+      </c>
+      <c r="K68" s="4">
+        <v>14</v>
+      </c>
+      <c r="L68" s="4">
+        <v>3</v>
+      </c>
       <c r="M68" s="4" t="s">
-        <v>460</v>
-      </c>
-      <c r="N68" s="4"/>
-      <c r="O68" s="4"/>
-      <c r="P68" s="4"/>
-      <c r="Q68" s="4"/>
+        <v>469</v>
+      </c>
+      <c r="N68" s="4">
+        <v>400</v>
+      </c>
+      <c r="O68" s="4">
+        <v>950</v>
+      </c>
+      <c r="P68" s="4">
+        <v>380</v>
+      </c>
+      <c r="Q68" s="4">
+        <v>93.5</v>
+      </c>
       <c r="R68" s="4" t="s">
-        <v>461</v>
-      </c>
-      <c r="S68" s="4"/>
-      <c r="T68" s="4"/>
-      <c r="U68" s="4"/>
-      <c r="V68" s="4"/>
-      <c r="W68" s="4"/>
-      <c r="X68" s="4"/>
-      <c r="Y68" s="4"/>
-      <c r="Z68" s="4"/>
-      <c r="AA68" s="4"/>
-      <c r="AB68" s="4"/>
-      <c r="AC68" s="4"/>
+        <v>470</v>
+      </c>
+      <c r="S68" s="4">
+        <v>26</v>
+      </c>
+      <c r="T68" s="4">
+        <v>28</v>
+      </c>
+      <c r="U68" s="4">
+        <v>2</v>
+      </c>
+      <c r="V68" s="4">
+        <v>0</v>
+      </c>
+      <c r="W68" s="4">
+        <v>1</v>
+      </c>
+      <c r="X68" s="4">
+        <v>9</v>
+      </c>
+      <c r="Y68" s="4">
+        <v>16</v>
+      </c>
+      <c r="Z68" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA68" s="4">
+        <v>14</v>
+      </c>
+      <c r="AB68" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC68" s="4" t="s">
+        <v>471</v>
+      </c>
     </row>
     <row r="69" spans="1:29" customHeight="1" ht="43.2">
       <c r="A69" s="4" t="s">
-        <v>462</v>
+        <v>472</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>463</v>
+        <v>473</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>33</v>
@@ -8144,7 +8576,7 @@
         <v>59</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>464</v>
+        <v>474</v>
       </c>
       <c r="F69" s="6">
         <v>20.439</v>
@@ -8153,42 +8585,78 @@
         <v>106.17400000000001</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>465</v>
+        <v>475</v>
       </c>
       <c r="I69" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="J69" s="4"/>
-      <c r="K69" s="4"/>
-      <c r="L69" s="4"/>
+      <c r="J69" s="4">
+        <v>8500</v>
+      </c>
+      <c r="K69" s="4">
+        <v>10</v>
+      </c>
+      <c r="L69" s="4">
+        <v>5</v>
+      </c>
       <c r="M69" s="4" t="s">
-        <v>466</v>
-      </c>
-      <c r="N69" s="4"/>
-      <c r="O69" s="4"/>
-      <c r="P69" s="4"/>
-      <c r="Q69" s="4"/>
+        <v>476</v>
+      </c>
+      <c r="N69" s="4">
+        <v>150</v>
+      </c>
+      <c r="O69" s="4">
+        <v>380</v>
+      </c>
+      <c r="P69" s="4">
+        <v>140</v>
+      </c>
+      <c r="Q69" s="4">
+        <v>94.0</v>
+      </c>
       <c r="R69" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="S69" s="4"/>
-      <c r="T69" s="4"/>
-      <c r="U69" s="4"/>
-      <c r="V69" s="4"/>
-      <c r="W69" s="4"/>
-      <c r="X69" s="4"/>
-      <c r="Y69" s="4"/>
-      <c r="Z69" s="4"/>
-      <c r="AA69" s="4"/>
-      <c r="AB69" s="4"/>
-      <c r="AC69" s="4"/>
+        <v>477</v>
+      </c>
+      <c r="S69" s="4">
+        <v>20</v>
+      </c>
+      <c r="T69" s="4">
+        <v>22</v>
+      </c>
+      <c r="U69" s="4">
+        <v>2</v>
+      </c>
+      <c r="V69" s="4">
+        <v>0</v>
+      </c>
+      <c r="W69" s="4">
+        <v>2</v>
+      </c>
+      <c r="X69" s="4">
+        <v>8</v>
+      </c>
+      <c r="Y69" s="4">
+        <v>10</v>
+      </c>
+      <c r="Z69" s="4">
+        <v>1</v>
+      </c>
+      <c r="AA69" s="4">
+        <v>12</v>
+      </c>
+      <c r="AB69" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC69" s="4" t="s">
+        <v>478</v>
+      </c>
     </row>
     <row r="70" spans="1:29" customHeight="1" ht="43.2">
       <c r="A70" s="4" t="s">
-        <v>468</v>
+        <v>479</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
       <c r="C70" s="4" t="s">
         <v>33</v>
@@ -8197,7 +8665,7 @@
         <v>265</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="F70" s="6">
         <v>20.3308</v>
@@ -8209,39 +8677,75 @@
         <v>61</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>471</v>
-      </c>
-      <c r="J70" s="4"/>
-      <c r="K70" s="4"/>
-      <c r="L70" s="4"/>
+        <v>482</v>
+      </c>
+      <c r="J70" s="4">
+        <v>17500</v>
+      </c>
+      <c r="K70" s="4">
+        <v>16</v>
+      </c>
+      <c r="L70" s="4">
+        <v>7</v>
+      </c>
       <c r="M70" s="4" t="s">
-        <v>472</v>
-      </c>
-      <c r="N70" s="4"/>
-      <c r="O70" s="4"/>
-      <c r="P70" s="4"/>
-      <c r="Q70" s="4"/>
+        <v>483</v>
+      </c>
+      <c r="N70" s="4">
+        <v>200</v>
+      </c>
+      <c r="O70" s="4">
+        <v>520</v>
+      </c>
+      <c r="P70" s="4">
+        <v>190</v>
+      </c>
+      <c r="Q70" s="4">
+        <v>96.0</v>
+      </c>
       <c r="R70" s="4" t="s">
-        <v>473</v>
-      </c>
-      <c r="S70" s="4"/>
-      <c r="T70" s="4"/>
-      <c r="U70" s="4"/>
-      <c r="V70" s="4"/>
-      <c r="W70" s="4"/>
-      <c r="X70" s="4"/>
-      <c r="Y70" s="4"/>
-      <c r="Z70" s="4"/>
-      <c r="AA70" s="4"/>
-      <c r="AB70" s="4"/>
-      <c r="AC70" s="4"/>
+        <v>484</v>
+      </c>
+      <c r="S70" s="4">
+        <v>28</v>
+      </c>
+      <c r="T70" s="4">
+        <v>30</v>
+      </c>
+      <c r="U70" s="4">
+        <v>2</v>
+      </c>
+      <c r="V70" s="4">
+        <v>0</v>
+      </c>
+      <c r="W70" s="4">
+        <v>2</v>
+      </c>
+      <c r="X70" s="4">
+        <v>11</v>
+      </c>
+      <c r="Y70" s="4">
+        <v>15</v>
+      </c>
+      <c r="Z70" s="4">
+        <v>1</v>
+      </c>
+      <c r="AA70" s="4">
+        <v>15</v>
+      </c>
+      <c r="AB70" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC70" s="4" t="s">
+        <v>485</v>
+      </c>
     </row>
     <row r="71" spans="1:29" customHeight="1" ht="28.8">
       <c r="A71" s="4" t="s">
-        <v>474</v>
+        <v>486</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>475</v>
+        <v>487</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>33</v>
@@ -8250,7 +8754,7 @@
         <v>83</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>476</v>
+        <v>488</v>
       </c>
       <c r="F71" s="6">
         <v>20.406</v>
@@ -8264,37 +8768,73 @@
       <c r="I71" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J71" s="4"/>
-      <c r="K71" s="4"/>
-      <c r="L71" s="4"/>
+      <c r="J71" s="4">
+        <v>6200</v>
+      </c>
+      <c r="K71" s="4">
+        <v>12</v>
+      </c>
+      <c r="L71" s="4">
+        <v>4</v>
+      </c>
       <c r="M71" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="N71" s="4"/>
-      <c r="O71" s="4"/>
-      <c r="P71" s="4"/>
-      <c r="Q71" s="4"/>
+        <v>489</v>
+      </c>
+      <c r="N71" s="4">
+        <v>120</v>
+      </c>
+      <c r="O71" s="4">
+        <v>320</v>
+      </c>
+      <c r="P71" s="4">
+        <v>110</v>
+      </c>
+      <c r="Q71" s="4">
+        <v>92.5</v>
+      </c>
       <c r="R71" s="4" t="s">
-        <v>478</v>
-      </c>
-      <c r="S71" s="4"/>
-      <c r="T71" s="4"/>
-      <c r="U71" s="4"/>
-      <c r="V71" s="4"/>
-      <c r="W71" s="4"/>
-      <c r="X71" s="4"/>
-      <c r="Y71" s="4"/>
-      <c r="Z71" s="4"/>
-      <c r="AA71" s="4"/>
-      <c r="AB71" s="4"/>
-      <c r="AC71" s="4"/>
+        <v>490</v>
+      </c>
+      <c r="S71" s="4">
+        <v>19</v>
+      </c>
+      <c r="T71" s="4">
+        <v>20</v>
+      </c>
+      <c r="U71" s="4">
+        <v>1</v>
+      </c>
+      <c r="V71" s="4">
+        <v>0</v>
+      </c>
+      <c r="W71" s="4">
+        <v>1</v>
+      </c>
+      <c r="X71" s="4">
+        <v>7</v>
+      </c>
+      <c r="Y71" s="4">
+        <v>11</v>
+      </c>
+      <c r="Z71" s="4">
+        <v>1</v>
+      </c>
+      <c r="AA71" s="4">
+        <v>11</v>
+      </c>
+      <c r="AB71" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC71" s="4" t="s">
+        <v>491</v>
+      </c>
     </row>
     <row r="72" spans="1:29" customHeight="1" ht="28.8">
       <c r="A72" s="4" t="s">
-        <v>479</v>
+        <v>492</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>480</v>
+        <v>493</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>33</v>
@@ -8303,7 +8843,7 @@
         <v>59</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>481</v>
+        <v>494</v>
       </c>
       <c r="F72" s="6">
         <v>20.43</v>
@@ -8317,37 +8857,73 @@
       <c r="I72" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J72" s="4"/>
-      <c r="K72" s="4"/>
-      <c r="L72" s="4"/>
+      <c r="J72" s="4">
+        <v>5800</v>
+      </c>
+      <c r="K72" s="4">
+        <v>14</v>
+      </c>
+      <c r="L72" s="4">
+        <v>3</v>
+      </c>
       <c r="M72" s="4" t="s">
-        <v>482</v>
-      </c>
-      <c r="N72" s="4"/>
-      <c r="O72" s="4"/>
-      <c r="P72" s="4"/>
-      <c r="Q72" s="4"/>
+        <v>495</v>
+      </c>
+      <c r="N72" s="4">
+        <v>150</v>
+      </c>
+      <c r="O72" s="4">
+        <v>390</v>
+      </c>
+      <c r="P72" s="4">
+        <v>140</v>
+      </c>
+      <c r="Q72" s="4">
+        <v>93.0</v>
+      </c>
       <c r="R72" s="4" t="s">
-        <v>483</v>
-      </c>
-      <c r="S72" s="4"/>
-      <c r="T72" s="4"/>
-      <c r="U72" s="4"/>
-      <c r="V72" s="4"/>
-      <c r="W72" s="4"/>
-      <c r="X72" s="4"/>
-      <c r="Y72" s="4"/>
-      <c r="Z72" s="4"/>
-      <c r="AA72" s="4"/>
-      <c r="AB72" s="4"/>
-      <c r="AC72" s="4"/>
+        <v>496</v>
+      </c>
+      <c r="S72" s="4">
+        <v>22</v>
+      </c>
+      <c r="T72" s="4">
+        <v>23</v>
+      </c>
+      <c r="U72" s="4">
+        <v>1</v>
+      </c>
+      <c r="V72" s="4">
+        <v>0</v>
+      </c>
+      <c r="W72" s="4">
+        <v>2</v>
+      </c>
+      <c r="X72" s="4">
+        <v>9</v>
+      </c>
+      <c r="Y72" s="4">
+        <v>11</v>
+      </c>
+      <c r="Z72" s="4">
+        <v>1</v>
+      </c>
+      <c r="AA72" s="4">
+        <v>14</v>
+      </c>
+      <c r="AB72" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC72" s="4" t="s">
+        <v>497</v>
+      </c>
     </row>
     <row r="73" spans="1:29" customHeight="1" ht="28.8">
       <c r="A73" s="4" t="s">
-        <v>484</v>
+        <v>498</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>485</v>
+        <v>499</v>
       </c>
       <c r="C73" s="4" t="s">
         <v>33</v>
@@ -8356,7 +8932,7 @@
         <v>59</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="F73" s="6">
         <v>20.4285</v>
@@ -8370,37 +8946,73 @@
       <c r="I73" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J73" s="4"/>
-      <c r="K73" s="4"/>
-      <c r="L73" s="4"/>
+      <c r="J73" s="4">
+        <v>4800</v>
+      </c>
+      <c r="K73" s="4">
+        <v>10</v>
+      </c>
+      <c r="L73" s="4">
+        <v>4</v>
+      </c>
       <c r="M73" s="4" t="s">
-        <v>487</v>
-      </c>
-      <c r="N73" s="4"/>
-      <c r="O73" s="4"/>
-      <c r="P73" s="4"/>
-      <c r="Q73" s="4"/>
+        <v>501</v>
+      </c>
+      <c r="N73" s="4">
+        <v>100</v>
+      </c>
+      <c r="O73" s="4">
+        <v>270</v>
+      </c>
+      <c r="P73" s="4">
+        <v>95</v>
+      </c>
+      <c r="Q73" s="4">
+        <v>94.0</v>
+      </c>
       <c r="R73" s="4" t="s">
-        <v>488</v>
-      </c>
-      <c r="S73" s="4"/>
-      <c r="T73" s="4"/>
-      <c r="U73" s="4"/>
-      <c r="V73" s="4"/>
-      <c r="W73" s="4"/>
-      <c r="X73" s="4"/>
-      <c r="Y73" s="4"/>
-      <c r="Z73" s="4"/>
-      <c r="AA73" s="4"/>
-      <c r="AB73" s="4"/>
-      <c r="AC73" s="4"/>
+        <v>502</v>
+      </c>
+      <c r="S73" s="4">
+        <v>17</v>
+      </c>
+      <c r="T73" s="4">
+        <v>18</v>
+      </c>
+      <c r="U73" s="4">
+        <v>1</v>
+      </c>
+      <c r="V73" s="4">
+        <v>0</v>
+      </c>
+      <c r="W73" s="4">
+        <v>1</v>
+      </c>
+      <c r="X73" s="4">
+        <v>6</v>
+      </c>
+      <c r="Y73" s="4">
+        <v>10</v>
+      </c>
+      <c r="Z73" s="4">
+        <v>1</v>
+      </c>
+      <c r="AA73" s="4">
+        <v>10</v>
+      </c>
+      <c r="AB73" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC73" s="4" t="s">
+        <v>503</v>
+      </c>
     </row>
     <row r="74" spans="1:29" customHeight="1" ht="28.8">
       <c r="A74" s="4" t="s">
-        <v>489</v>
+        <v>504</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>490</v>
+        <v>505</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>33</v>
@@ -8409,7 +9021,7 @@
         <v>144</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>491</v>
+        <v>506</v>
       </c>
       <c r="F74" s="6">
         <v>20.4</v>
@@ -8423,46 +9035,82 @@
       <c r="I74" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J74" s="4"/>
-      <c r="K74" s="4"/>
-      <c r="L74" s="4"/>
+      <c r="J74" s="4">
+        <v>16500</v>
+      </c>
+      <c r="K74" s="4">
+        <v>12</v>
+      </c>
+      <c r="L74" s="4">
+        <v>5</v>
+      </c>
       <c r="M74" s="4" t="s">
-        <v>492</v>
-      </c>
-      <c r="N74" s="4"/>
-      <c r="O74" s="4"/>
-      <c r="P74" s="4"/>
-      <c r="Q74" s="4"/>
+        <v>507</v>
+      </c>
+      <c r="N74" s="4">
+        <v>120</v>
+      </c>
+      <c r="O74" s="4">
+        <v>310</v>
+      </c>
+      <c r="P74" s="4">
+        <v>112</v>
+      </c>
+      <c r="Q74" s="4">
+        <v>91.5</v>
+      </c>
       <c r="R74" s="4" t="s">
-        <v>493</v>
-      </c>
-      <c r="S74" s="4"/>
-      <c r="T74" s="4"/>
-      <c r="U74" s="4"/>
-      <c r="V74" s="4"/>
-      <c r="W74" s="4"/>
-      <c r="X74" s="4"/>
-      <c r="Y74" s="4"/>
-      <c r="Z74" s="4"/>
-      <c r="AA74" s="4"/>
-      <c r="AB74" s="4"/>
-      <c r="AC74" s="4"/>
+        <v>508</v>
+      </c>
+      <c r="S74" s="4">
+        <v>19</v>
+      </c>
+      <c r="T74" s="4">
+        <v>21</v>
+      </c>
+      <c r="U74" s="4">
+        <v>2</v>
+      </c>
+      <c r="V74" s="4">
+        <v>0</v>
+      </c>
+      <c r="W74" s="4">
+        <v>1</v>
+      </c>
+      <c r="X74" s="4">
+        <v>7</v>
+      </c>
+      <c r="Y74" s="4">
+        <v>11</v>
+      </c>
+      <c r="Z74" s="4">
+        <v>1</v>
+      </c>
+      <c r="AA74" s="4">
+        <v>11</v>
+      </c>
+      <c r="AB74" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC74" s="4" t="s">
+        <v>509</v>
+      </c>
     </row>
     <row r="75" spans="1:29" customHeight="1" ht="28.8">
       <c r="A75" s="4" t="s">
-        <v>494</v>
+        <v>510</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>495</v>
+        <v>511</v>
       </c>
       <c r="C75" s="4" t="s">
         <v>33</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>496</v>
+        <v>512</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>497</v>
+        <v>513</v>
       </c>
       <c r="F75" s="6">
         <v>20.25</v>
@@ -8476,46 +9124,82 @@
       <c r="I75" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J75" s="4"/>
-      <c r="K75" s="4"/>
-      <c r="L75" s="4"/>
+      <c r="J75" s="4">
+        <v>8900</v>
+      </c>
+      <c r="K75" s="4">
+        <v>11</v>
+      </c>
+      <c r="L75" s="4">
+        <v>4</v>
+      </c>
       <c r="M75" s="4" t="s">
-        <v>498</v>
-      </c>
-      <c r="N75" s="4"/>
-      <c r="O75" s="4"/>
-      <c r="P75" s="4"/>
-      <c r="Q75" s="4"/>
+        <v>514</v>
+      </c>
+      <c r="N75" s="4">
+        <v>100</v>
+      </c>
+      <c r="O75" s="4">
+        <v>260</v>
+      </c>
+      <c r="P75" s="4">
+        <v>94</v>
+      </c>
+      <c r="Q75" s="4">
+        <v>92.0</v>
+      </c>
       <c r="R75" s="4" t="s">
-        <v>499</v>
-      </c>
-      <c r="S75" s="4"/>
-      <c r="T75" s="4"/>
-      <c r="U75" s="4"/>
-      <c r="V75" s="4"/>
-      <c r="W75" s="4"/>
-      <c r="X75" s="4"/>
-      <c r="Y75" s="4"/>
-      <c r="Z75" s="4"/>
-      <c r="AA75" s="4"/>
-      <c r="AB75" s="4"/>
-      <c r="AC75" s="4"/>
+        <v>515</v>
+      </c>
+      <c r="S75" s="4">
+        <v>16</v>
+      </c>
+      <c r="T75" s="4">
+        <v>18</v>
+      </c>
+      <c r="U75" s="4">
+        <v>2</v>
+      </c>
+      <c r="V75" s="4">
+        <v>0</v>
+      </c>
+      <c r="W75" s="4">
+        <v>1</v>
+      </c>
+      <c r="X75" s="4">
+        <v>6</v>
+      </c>
+      <c r="Y75" s="4">
+        <v>9</v>
+      </c>
+      <c r="Z75" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA75" s="4">
+        <v>9</v>
+      </c>
+      <c r="AB75" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC75" s="4" t="s">
+        <v>516</v>
+      </c>
     </row>
     <row r="76" spans="1:29" customHeight="1" ht="28.8">
       <c r="A76" s="4" t="s">
-        <v>500</v>
+        <v>517</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>501</v>
+        <v>518</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>33</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>502</v>
+        <v>519</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>503</v>
+        <v>520</v>
       </c>
       <c r="F76" s="6">
         <v>20.257</v>
@@ -8529,37 +9213,73 @@
       <c r="I76" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J76" s="4"/>
-      <c r="K76" s="4"/>
-      <c r="L76" s="4"/>
+      <c r="J76" s="4">
+        <v>7800</v>
+      </c>
+      <c r="K76" s="4">
+        <v>10</v>
+      </c>
+      <c r="L76" s="4">
+        <v>4</v>
+      </c>
       <c r="M76" s="4" t="s">
-        <v>504</v>
-      </c>
-      <c r="N76" s="4"/>
-      <c r="O76" s="4"/>
-      <c r="P76" s="4"/>
-      <c r="Q76" s="4"/>
+        <v>521</v>
+      </c>
+      <c r="N76" s="4">
+        <v>100</v>
+      </c>
+      <c r="O76" s="4">
+        <v>255</v>
+      </c>
+      <c r="P76" s="4">
+        <v>92</v>
+      </c>
+      <c r="Q76" s="4">
+        <v>93.5</v>
+      </c>
       <c r="R76" s="4" t="s">
-        <v>505</v>
-      </c>
-      <c r="S76" s="4"/>
-      <c r="T76" s="4"/>
-      <c r="U76" s="4"/>
-      <c r="V76" s="4"/>
-      <c r="W76" s="4"/>
-      <c r="X76" s="4"/>
-      <c r="Y76" s="4"/>
-      <c r="Z76" s="4"/>
-      <c r="AA76" s="4"/>
-      <c r="AB76" s="4"/>
-      <c r="AC76" s="4"/>
+        <v>522</v>
+      </c>
+      <c r="S76" s="4">
+        <v>15</v>
+      </c>
+      <c r="T76" s="4">
+        <v>16</v>
+      </c>
+      <c r="U76" s="4">
+        <v>1</v>
+      </c>
+      <c r="V76" s="4">
+        <v>0</v>
+      </c>
+      <c r="W76" s="4">
+        <v>1</v>
+      </c>
+      <c r="X76" s="4">
+        <v>5</v>
+      </c>
+      <c r="Y76" s="4">
+        <v>9</v>
+      </c>
+      <c r="Z76" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="4">
+        <v>8</v>
+      </c>
+      <c r="AB76" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC76" s="4" t="s">
+        <v>523</v>
+      </c>
     </row>
     <row r="77" spans="1:29" customHeight="1" ht="28.8">
       <c r="A77" s="4" t="s">
-        <v>506</v>
+        <v>524</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>507</v>
+        <v>525</v>
       </c>
       <c r="C77" s="4" t="s">
         <v>33</v>
@@ -8568,7 +9288,7 @@
         <v>271</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>508</v>
+        <v>526</v>
       </c>
       <c r="F77" s="6">
         <v>20.33</v>
@@ -8582,37 +9302,73 @@
       <c r="I77" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J77" s="4"/>
-      <c r="K77" s="4"/>
-      <c r="L77" s="4"/>
+      <c r="J77" s="4">
+        <v>11500</v>
+      </c>
+      <c r="K77" s="4">
+        <v>12</v>
+      </c>
+      <c r="L77" s="4">
+        <v>5</v>
+      </c>
       <c r="M77" s="4" t="s">
-        <v>509</v>
-      </c>
-      <c r="N77" s="4"/>
-      <c r="O77" s="4"/>
-      <c r="P77" s="4"/>
-      <c r="Q77" s="4"/>
+        <v>527</v>
+      </c>
+      <c r="N77" s="4">
+        <v>120</v>
+      </c>
+      <c r="O77" s="4">
+        <v>315</v>
+      </c>
+      <c r="P77" s="4">
+        <v>115</v>
+      </c>
+      <c r="Q77" s="4">
+        <v>95.0</v>
+      </c>
       <c r="R77" s="4" t="s">
-        <v>510</v>
-      </c>
-      <c r="S77" s="4"/>
-      <c r="T77" s="4"/>
-      <c r="U77" s="4"/>
-      <c r="V77" s="4"/>
-      <c r="W77" s="4"/>
-      <c r="X77" s="4"/>
-      <c r="Y77" s="4"/>
-      <c r="Z77" s="4"/>
-      <c r="AA77" s="4"/>
-      <c r="AB77" s="4"/>
-      <c r="AC77" s="4"/>
+        <v>528</v>
+      </c>
+      <c r="S77" s="4">
+        <v>18</v>
+      </c>
+      <c r="T77" s="4">
+        <v>20</v>
+      </c>
+      <c r="U77" s="4">
+        <v>2</v>
+      </c>
+      <c r="V77" s="4">
+        <v>0</v>
+      </c>
+      <c r="W77" s="4">
+        <v>1</v>
+      </c>
+      <c r="X77" s="4">
+        <v>7</v>
+      </c>
+      <c r="Y77" s="4">
+        <v>10</v>
+      </c>
+      <c r="Z77" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="4">
+        <v>9</v>
+      </c>
+      <c r="AB77" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC77" s="4" t="s">
+        <v>529</v>
+      </c>
     </row>
     <row r="78" spans="1:29" customHeight="1" ht="28.8">
       <c r="A78" s="4" t="s">
-        <v>511</v>
+        <v>530</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>512</v>
+        <v>531</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>33</v>
@@ -8621,7 +9377,7 @@
         <v>271</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>513</v>
+        <v>532</v>
       </c>
       <c r="F78" s="6">
         <v>20.315</v>
@@ -8635,37 +9391,73 @@
       <c r="I78" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J78" s="4"/>
-      <c r="K78" s="4"/>
-      <c r="L78" s="4"/>
+      <c r="J78" s="4">
+        <v>7200</v>
+      </c>
+      <c r="K78" s="4">
+        <v>10</v>
+      </c>
+      <c r="L78" s="4">
+        <v>3</v>
+      </c>
       <c r="M78" s="4" t="s">
-        <v>514</v>
-      </c>
-      <c r="N78" s="4"/>
-      <c r="O78" s="4"/>
-      <c r="P78" s="4"/>
-      <c r="Q78" s="4"/>
+        <v>533</v>
+      </c>
+      <c r="N78" s="4">
+        <v>90</v>
+      </c>
+      <c r="O78" s="4">
+        <v>230</v>
+      </c>
+      <c r="P78" s="4">
+        <v>85</v>
+      </c>
+      <c r="Q78" s="4">
+        <v>91.0</v>
+      </c>
       <c r="R78" s="4" t="s">
-        <v>515</v>
-      </c>
-      <c r="S78" s="4"/>
-      <c r="T78" s="4"/>
-      <c r="U78" s="4"/>
-      <c r="V78" s="4"/>
-      <c r="W78" s="4"/>
-      <c r="X78" s="4"/>
-      <c r="Y78" s="4"/>
-      <c r="Z78" s="4"/>
-      <c r="AA78" s="4"/>
-      <c r="AB78" s="4"/>
-      <c r="AC78" s="4"/>
+        <v>534</v>
+      </c>
+      <c r="S78" s="4">
+        <v>14</v>
+      </c>
+      <c r="T78" s="4">
+        <v>15</v>
+      </c>
+      <c r="U78" s="4">
+        <v>1</v>
+      </c>
+      <c r="V78" s="4">
+        <v>0</v>
+      </c>
+      <c r="W78" s="4">
+        <v>1</v>
+      </c>
+      <c r="X78" s="4">
+        <v>5</v>
+      </c>
+      <c r="Y78" s="4">
+        <v>8</v>
+      </c>
+      <c r="Z78" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="4">
+        <v>7</v>
+      </c>
+      <c r="AB78" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC78" s="4" t="s">
+        <v>535</v>
+      </c>
     </row>
     <row r="79" spans="1:29" customHeight="1" ht="28.8">
       <c r="A79" s="4" t="s">
-        <v>516</v>
+        <v>536</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>517</v>
+        <v>537</v>
       </c>
       <c r="C79" s="4" t="s">
         <v>33</v>
@@ -8674,7 +9466,7 @@
         <v>144</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>518</v>
+        <v>538</v>
       </c>
       <c r="F79" s="6">
         <v>20.405</v>
@@ -8688,37 +9480,73 @@
       <c r="I79" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J79" s="4"/>
-      <c r="K79" s="4"/>
-      <c r="L79" s="4"/>
+      <c r="J79" s="4">
+        <v>5100</v>
+      </c>
+      <c r="K79" s="4">
+        <v>8</v>
+      </c>
+      <c r="L79" s="4">
+        <v>3</v>
+      </c>
       <c r="M79" s="4" t="s">
-        <v>519</v>
-      </c>
-      <c r="N79" s="4"/>
-      <c r="O79" s="4"/>
-      <c r="P79" s="4"/>
-      <c r="Q79" s="4"/>
+        <v>539</v>
+      </c>
+      <c r="N79" s="4">
+        <v>80</v>
+      </c>
+      <c r="O79" s="4">
+        <v>210</v>
+      </c>
+      <c r="P79" s="4">
+        <v>75</v>
+      </c>
+      <c r="Q79" s="4">
+        <v>93.0</v>
+      </c>
       <c r="R79" s="4" t="s">
-        <v>520</v>
-      </c>
-      <c r="S79" s="4"/>
-      <c r="T79" s="4"/>
-      <c r="U79" s="4"/>
-      <c r="V79" s="4"/>
-      <c r="W79" s="4"/>
-      <c r="X79" s="4"/>
-      <c r="Y79" s="4"/>
-      <c r="Z79" s="4"/>
-      <c r="AA79" s="4"/>
-      <c r="AB79" s="4"/>
-      <c r="AC79" s="4"/>
+        <v>540</v>
+      </c>
+      <c r="S79" s="4">
+        <v>13</v>
+      </c>
+      <c r="T79" s="4">
+        <v>14</v>
+      </c>
+      <c r="U79" s="4">
+        <v>1</v>
+      </c>
+      <c r="V79" s="4">
+        <v>0</v>
+      </c>
+      <c r="W79" s="4">
+        <v>1</v>
+      </c>
+      <c r="X79" s="4">
+        <v>4</v>
+      </c>
+      <c r="Y79" s="4">
+        <v>8</v>
+      </c>
+      <c r="Z79" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="4">
+        <v>6</v>
+      </c>
+      <c r="AB79" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC79" s="4" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="80" spans="1:29" customHeight="1" ht="28.8">
       <c r="A80" s="4" t="s">
-        <v>521</v>
+        <v>542</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>522</v>
+        <v>543</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>33</v>
@@ -8727,7 +9555,7 @@
         <v>380</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>523</v>
+        <v>544</v>
       </c>
       <c r="F80" s="6">
         <v>20.28</v>
@@ -8741,37 +9569,73 @@
       <c r="I80" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J80" s="4"/>
-      <c r="K80" s="4"/>
-      <c r="L80" s="4"/>
+      <c r="J80" s="4">
+        <v>10500</v>
+      </c>
+      <c r="K80" s="4">
+        <v>12</v>
+      </c>
+      <c r="L80" s="4">
+        <v>4</v>
+      </c>
       <c r="M80" s="4" t="s">
-        <v>524</v>
-      </c>
-      <c r="N80" s="4"/>
-      <c r="O80" s="4"/>
-      <c r="P80" s="4"/>
-      <c r="Q80" s="4"/>
+        <v>545</v>
+      </c>
+      <c r="N80" s="4">
+        <v>120</v>
+      </c>
+      <c r="O80" s="4">
+        <v>320</v>
+      </c>
+      <c r="P80" s="4">
+        <v>110</v>
+      </c>
+      <c r="Q80" s="4">
+        <v>92.5</v>
+      </c>
       <c r="R80" s="4" t="s">
-        <v>525</v>
-      </c>
-      <c r="S80" s="4"/>
-      <c r="T80" s="4"/>
-      <c r="U80" s="4"/>
-      <c r="V80" s="4"/>
-      <c r="W80" s="4"/>
-      <c r="X80" s="4"/>
-      <c r="Y80" s="4"/>
-      <c r="Z80" s="4"/>
-      <c r="AA80" s="4"/>
-      <c r="AB80" s="4"/>
-      <c r="AC80" s="4"/>
+        <v>546</v>
+      </c>
+      <c r="S80" s="4">
+        <v>18</v>
+      </c>
+      <c r="T80" s="4">
+        <v>19</v>
+      </c>
+      <c r="U80" s="4">
+        <v>1</v>
+      </c>
+      <c r="V80" s="4">
+        <v>0</v>
+      </c>
+      <c r="W80" s="4">
+        <v>1</v>
+      </c>
+      <c r="X80" s="4">
+        <v>6</v>
+      </c>
+      <c r="Y80" s="4">
+        <v>11</v>
+      </c>
+      <c r="Z80" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="4">
+        <v>9</v>
+      </c>
+      <c r="AB80" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC80" s="4" t="s">
+        <v>547</v>
+      </c>
     </row>
     <row r="81" spans="1:29" customHeight="1" ht="28.8">
       <c r="A81" s="4" t="s">
-        <v>526</v>
+        <v>548</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>527</v>
+        <v>549</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>209</v>
@@ -8780,7 +9644,7 @@
         <v>238</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>528</v>
+        <v>550</v>
       </c>
       <c r="F81" s="6">
         <v>20.1958125</v>
@@ -8794,46 +9658,82 @@
       <c r="I81" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="J81" s="4"/>
-      <c r="K81" s="4"/>
-      <c r="L81" s="4"/>
+      <c r="J81" s="4">
+        <v>12800</v>
+      </c>
+      <c r="K81" s="4">
+        <v>15</v>
+      </c>
+      <c r="L81" s="4">
+        <v>5</v>
+      </c>
       <c r="M81" s="4" t="s">
-        <v>529</v>
-      </c>
-      <c r="N81" s="4"/>
-      <c r="O81" s="4"/>
-      <c r="P81" s="4"/>
-      <c r="Q81" s="4"/>
+        <v>551</v>
+      </c>
+      <c r="N81" s="4">
+        <v>270</v>
+      </c>
+      <c r="O81" s="4">
+        <v>740</v>
+      </c>
+      <c r="P81" s="4">
+        <v>250</v>
+      </c>
+      <c r="Q81" s="4">
+        <v>90.5</v>
+      </c>
       <c r="R81" s="4" t="s">
-        <v>530</v>
-      </c>
-      <c r="S81" s="4"/>
-      <c r="T81" s="4"/>
-      <c r="U81" s="4"/>
-      <c r="V81" s="4"/>
-      <c r="W81" s="4"/>
-      <c r="X81" s="4"/>
-      <c r="Y81" s="4"/>
-      <c r="Z81" s="4"/>
-      <c r="AA81" s="4"/>
-      <c r="AB81" s="4"/>
-      <c r="AC81" s="4"/>
+        <v>552</v>
+      </c>
+      <c r="S81" s="4">
+        <v>24</v>
+      </c>
+      <c r="T81" s="4">
+        <v>26</v>
+      </c>
+      <c r="U81" s="4">
+        <v>2</v>
+      </c>
+      <c r="V81" s="4">
+        <v>0</v>
+      </c>
+      <c r="W81" s="4">
+        <v>0</v>
+      </c>
+      <c r="X81" s="4">
+        <v>8</v>
+      </c>
+      <c r="Y81" s="4">
+        <v>16</v>
+      </c>
+      <c r="Z81" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="4">
+        <v>9</v>
+      </c>
+      <c r="AB81" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC81" s="4" t="s">
+        <v>553</v>
+      </c>
     </row>
     <row r="82" spans="1:29">
       <c r="A82" s="4" t="s">
-        <v>531</v>
+        <v>554</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>532</v>
+        <v>555</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>209</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>533</v>
+        <v>556</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>534</v>
+        <v>557</v>
       </c>
       <c r="F82" s="6">
         <v>20.2063375</v>
@@ -8847,30 +9747,66 @@
       <c r="I82" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="J82" s="4"/>
-      <c r="K82" s="4"/>
-      <c r="L82" s="4"/>
+      <c r="J82" s="4">
+        <v>8700</v>
+      </c>
+      <c r="K82" s="4">
+        <v>11</v>
+      </c>
+      <c r="L82" s="4">
+        <v>3</v>
+      </c>
       <c r="M82" s="4" t="s">
-        <v>535</v>
-      </c>
-      <c r="N82" s="4"/>
-      <c r="O82" s="4"/>
-      <c r="P82" s="4"/>
-      <c r="Q82" s="4"/>
+        <v>558</v>
+      </c>
+      <c r="N82" s="4">
+        <v>200</v>
+      </c>
+      <c r="O82" s="4">
+        <v>550</v>
+      </c>
+      <c r="P82" s="4">
+        <v>185</v>
+      </c>
+      <c r="Q82" s="4">
+        <v>89.0</v>
+      </c>
       <c r="R82" s="4" t="s">
-        <v>536</v>
-      </c>
-      <c r="S82" s="4"/>
-      <c r="T82" s="4"/>
-      <c r="U82" s="4"/>
-      <c r="V82" s="4"/>
-      <c r="W82" s="4"/>
-      <c r="X82" s="4"/>
-      <c r="Y82" s="4"/>
-      <c r="Z82" s="4"/>
-      <c r="AA82" s="4"/>
-      <c r="AB82" s="4"/>
-      <c r="AC82" s="4"/>
+        <v>559</v>
+      </c>
+      <c r="S82" s="4">
+        <v>19</v>
+      </c>
+      <c r="T82" s="4">
+        <v>20</v>
+      </c>
+      <c r="U82" s="4">
+        <v>1</v>
+      </c>
+      <c r="V82" s="4">
+        <v>0</v>
+      </c>
+      <c r="W82" s="4">
+        <v>0</v>
+      </c>
+      <c r="X82" s="4">
+        <v>6</v>
+      </c>
+      <c r="Y82" s="4">
+        <v>13</v>
+      </c>
+      <c r="Z82" s="4">
+        <v>0</v>
+      </c>
+      <c r="AA82" s="4">
+        <v>7</v>
+      </c>
+      <c r="AB82" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC82" s="4" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="83" spans="1:29">
       <c r="A83" s="4"/>
@@ -9007,361 +9943,361 @@
   <sheetData>
     <row r="1" spans="1:3" customHeight="1" ht="30">
       <c r="A1" s="9" t="s">
-        <v>537</v>
+        <v>561</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
     </row>
     <row r="3" spans="1:3" customHeight="1" ht="28.05">
       <c r="A3" s="1" t="s">
-        <v>538</v>
+        <v>562</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>539</v>
+        <v>563</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>540</v>
+        <v>564</v>
       </c>
     </row>
     <row r="4" spans="1:3" customHeight="1" ht="24">
       <c r="A4" s="3" t="s">
-        <v>541</v>
+        <v>565</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>542</v>
+        <v>566</v>
       </c>
     </row>
     <row r="5" spans="1:3" customHeight="1" ht="24">
       <c r="A5" s="3" t="s">
-        <v>543</v>
+        <v>567</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>544</v>
+        <v>568</v>
       </c>
     </row>
     <row r="6" spans="1:3" customHeight="1" ht="24">
       <c r="A6" s="3" t="s">
-        <v>545</v>
+        <v>569</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>546</v>
+        <v>570</v>
       </c>
     </row>
     <row r="7" spans="1:3" customHeight="1" ht="24">
       <c r="A7" s="3" t="s">
-        <v>547</v>
+        <v>571</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>548</v>
+        <v>572</v>
       </c>
     </row>
     <row r="8" spans="1:3" customHeight="1" ht="24">
       <c r="A8" s="3" t="s">
-        <v>549</v>
+        <v>573</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>550</v>
+        <v>574</v>
       </c>
     </row>
     <row r="9" spans="1:3" customHeight="1" ht="24">
       <c r="A9" s="3" t="s">
-        <v>551</v>
+        <v>575</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>552</v>
+        <v>576</v>
       </c>
     </row>
     <row r="10" spans="1:3" customHeight="1" ht="24">
       <c r="A10" s="3" t="s">
-        <v>553</v>
+        <v>577</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>554</v>
+        <v>578</v>
       </c>
     </row>
     <row r="11" spans="1:3" customHeight="1" ht="24">
       <c r="A11" s="3" t="s">
-        <v>555</v>
+        <v>579</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>556</v>
+        <v>580</v>
       </c>
     </row>
     <row r="12" spans="1:3" customHeight="1" ht="24">
       <c r="A12" s="3" t="s">
-        <v>557</v>
+        <v>581</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>558</v>
+        <v>582</v>
       </c>
     </row>
     <row r="13" spans="1:3" customHeight="1" ht="24">
       <c r="A13" s="3" t="s">
-        <v>559</v>
+        <v>583</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>560</v>
+        <v>584</v>
       </c>
     </row>
     <row r="14" spans="1:3" customHeight="1" ht="24">
       <c r="A14" s="3" t="s">
-        <v>561</v>
+        <v>585</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>562</v>
+        <v>586</v>
       </c>
     </row>
     <row r="15" spans="1:3" customHeight="1" ht="24">
       <c r="A15" s="3" t="s">
-        <v>563</v>
+        <v>587</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>564</v>
+        <v>588</v>
       </c>
     </row>
     <row r="16" spans="1:3" customHeight="1" ht="24">
       <c r="A16" s="3" t="s">
-        <v>565</v>
+        <v>589</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>566</v>
+        <v>590</v>
       </c>
     </row>
     <row r="17" spans="1:3" customHeight="1" ht="24">
       <c r="A17" s="3" t="s">
-        <v>567</v>
+        <v>591</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>568</v>
+        <v>592</v>
       </c>
     </row>
     <row r="18" spans="1:3" customHeight="1" ht="24">
       <c r="A18" s="3" t="s">
-        <v>569</v>
+        <v>593</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>570</v>
+        <v>594</v>
       </c>
     </row>
     <row r="19" spans="1:3" customHeight="1" ht="24">
       <c r="A19" s="3" t="s">
-        <v>571</v>
+        <v>595</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>572</v>
+        <v>596</v>
       </c>
     </row>
     <row r="20" spans="1:3" customHeight="1" ht="24">
       <c r="A20" s="3" t="s">
-        <v>573</v>
+        <v>597</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>574</v>
+        <v>598</v>
       </c>
     </row>
     <row r="21" spans="1:3" customHeight="1" ht="24">
       <c r="A21" s="3" t="s">
-        <v>575</v>
+        <v>599</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>576</v>
+        <v>600</v>
       </c>
     </row>
     <row r="22" spans="1:3" customHeight="1" ht="24">
       <c r="A22" s="3" t="s">
-        <v>577</v>
+        <v>601</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>578</v>
+        <v>602</v>
       </c>
     </row>
     <row r="23" spans="1:3" customHeight="1" ht="24">
       <c r="A23" s="3" t="s">
-        <v>579</v>
+        <v>603</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>580</v>
+        <v>604</v>
       </c>
     </row>
     <row r="24" spans="1:3" customHeight="1" ht="24">
       <c r="A24" s="3" t="s">
-        <v>581</v>
+        <v>605</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>582</v>
+        <v>606</v>
       </c>
     </row>
     <row r="25" spans="1:3" customHeight="1" ht="24">
       <c r="A25" s="3" t="s">
-        <v>583</v>
+        <v>607</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>584</v>
+        <v>608</v>
       </c>
     </row>
     <row r="26" spans="1:3" customHeight="1" ht="24">
       <c r="A26" s="3" t="s">
-        <v>585</v>
+        <v>609</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>586</v>
+        <v>610</v>
       </c>
     </row>
     <row r="27" spans="1:3" customHeight="1" ht="24">
       <c r="A27" s="3" t="s">
-        <v>587</v>
+        <v>611</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>588</v>
+        <v>612</v>
       </c>
     </row>
     <row r="28" spans="1:3" customHeight="1" ht="24">
       <c r="A28" s="3" t="s">
-        <v>589</v>
+        <v>613</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>590</v>
+        <v>614</v>
       </c>
     </row>
     <row r="29" spans="1:3" customHeight="1" ht="24">
       <c r="A29" s="3" t="s">
-        <v>591</v>
+        <v>615</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>592</v>
+        <v>616</v>
       </c>
     </row>
     <row r="30" spans="1:3" customHeight="1" ht="24">
       <c r="A30" s="3" t="s">
-        <v>593</v>
+        <v>617</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>594</v>
+        <v>618</v>
       </c>
     </row>
     <row r="31" spans="1:3" customHeight="1" ht="24">
       <c r="A31" s="3" t="s">
-        <v>595</v>
+        <v>619</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>30</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>596</v>
+        <v>620</v>
       </c>
     </row>
     <row r="33" spans="1:3" customHeight="1" ht="43.2">
       <c r="A33" s="5" t="s">
-        <v>597</v>
+        <v>621</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
     </row>
     <row r="34" spans="1:3" customHeight="1" ht="43.2">
       <c r="A34" s="4" t="s">
-        <v>598</v>
+        <v>622</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>599</v>
+        <v>623</v>
       </c>
       <c r="C34" s="4"/>
     </row>
     <row r="35" spans="1:3" customHeight="1" ht="57.6">
       <c r="A35" s="4" t="s">
-        <v>600</v>
+        <v>624</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>601</v>
+        <v>625</v>
       </c>
       <c r="C35" s="4"/>
     </row>
     <row r="36" spans="1:3" customHeight="1" ht="57.6">
       <c r="A36" s="4" t="s">
-        <v>602</v>
+        <v>626</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>603</v>
+        <v>627</v>
       </c>
       <c r="C36" s="4"/>
     </row>
@@ -9389,18 +10325,18 @@
   <sheetData>
     <row r="1" spans="1:2" customHeight="1" ht="28.05">
       <c r="A1" s="1" t="s">
-        <v>604</v>
+        <v>628</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>605</v>
+        <v>629</v>
       </c>
     </row>
     <row r="2" spans="1:2" customHeight="1" ht="22.05">
       <c r="A2" s="2" t="s">
-        <v>606</v>
+        <v>630</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>607</v>
+        <v>631</v>
       </c>
     </row>
     <row r="3" spans="1:2" customHeight="1" ht="22.05">
@@ -9408,7 +10344,7 @@
         <v>33</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>608</v>
+        <v>632</v>
       </c>
     </row>
     <row r="4" spans="1:2" customHeight="1" ht="22.05">
@@ -9416,7 +10352,7 @@
         <v>143</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>609</v>
+        <v>633</v>
       </c>
     </row>
     <row r="5" spans="1:2" customHeight="1" ht="22.05">
@@ -9437,12 +10373,12 @@
     </row>
     <row r="7" spans="1:2" customHeight="1" ht="22.05">
       <c r="B7" s="2" t="s">
-        <v>610</v>
+        <v>634</v>
       </c>
     </row>
     <row r="8" spans="1:2" customHeight="1" ht="22.05">
       <c r="B8" s="2" t="s">
-        <v>611</v>
+        <v>635</v>
       </c>
     </row>
     <row r="9" spans="1:2" customHeight="1" ht="22.05">
@@ -9457,7 +10393,7 @@
     </row>
     <row r="11" spans="1:2" customHeight="1" ht="22.05">
       <c r="B11" s="2" t="s">
-        <v>612</v>
+        <v>636</v>
       </c>
     </row>
     <row r="12" spans="1:2" customHeight="1" ht="22.05">
@@ -9467,22 +10403,22 @@
     </row>
     <row r="13" spans="1:2" customHeight="1" ht="22.05">
       <c r="B13" s="2" t="s">
-        <v>613</v>
+        <v>637</v>
       </c>
     </row>
     <row r="14" spans="1:2" customHeight="1" ht="22.05">
       <c r="B14" s="2" t="s">
-        <v>614</v>
+        <v>638</v>
       </c>
     </row>
     <row r="15" spans="1:2" customHeight="1" ht="22.05">
       <c r="B15" s="2" t="s">
-        <v>615</v>
+        <v>639</v>
       </c>
     </row>
     <row r="16" spans="1:2" customHeight="1" ht="22.05">
       <c r="B16" s="2" t="s">
-        <v>616</v>
+        <v>640</v>
       </c>
     </row>
     <row r="17" spans="1:2" customHeight="1" ht="22.05">
@@ -9497,12 +10433,12 @@
     </row>
     <row r="19" spans="1:2" customHeight="1" ht="22.05">
       <c r="B19" s="2" t="s">
-        <v>617</v>
+        <v>641</v>
       </c>
     </row>
     <row r="20" spans="1:2" customHeight="1" ht="22.05">
       <c r="B20" s="2" t="s">
-        <v>618</v>
+        <v>642</v>
       </c>
     </row>
     <row r="21" spans="1:2" customHeight="1" ht="22.05">
@@ -9522,12 +10458,12 @@
     </row>
     <row r="24" spans="1:2" customHeight="1" ht="22.05">
       <c r="B24" s="2" t="s">
-        <v>619</v>
+        <v>643</v>
       </c>
     </row>
     <row r="25" spans="1:2" customHeight="1" ht="22.05">
       <c r="B25" s="2" t="s">
-        <v>620</v>
+        <v>644</v>
       </c>
     </row>
     <row r="26" spans="1:2" customHeight="1" ht="22.05">
@@ -9542,7 +10478,7 @@
     </row>
     <row r="28" spans="1:2" customHeight="1" ht="22.05">
       <c r="B28" s="2" t="s">
-        <v>621</v>
+        <v>645</v>
       </c>
     </row>
     <row r="29" spans="1:2" customHeight="1" ht="22.05">
@@ -9572,27 +10508,27 @@
     </row>
     <row r="34" spans="1:2" customHeight="1" ht="22.05">
       <c r="B34" s="2" t="s">
-        <v>622</v>
+        <v>646</v>
       </c>
     </row>
     <row r="35" spans="1:2" customHeight="1" ht="22.05">
       <c r="B35" s="2" t="s">
-        <v>623</v>
+        <v>647</v>
       </c>
     </row>
     <row r="36" spans="1:2" customHeight="1" ht="22.05">
       <c r="B36" s="2" t="s">
-        <v>624</v>
+        <v>648</v>
       </c>
     </row>
     <row r="37" spans="1:2" customHeight="1" ht="22.05">
       <c r="B37" s="2" t="s">
-        <v>625</v>
+        <v>649</v>
       </c>
     </row>
     <row r="38" spans="1:2" customHeight="1" ht="22.05">
       <c r="B38" s="2" t="s">
-        <v>626</v>
+        <v>650</v>
       </c>
     </row>
     <row r="39" spans="1:2" customHeight="1" ht="22.05">
@@ -9602,17 +10538,17 @@
     </row>
     <row r="40" spans="1:2" customHeight="1" ht="22.05">
       <c r="B40" s="2" t="s">
-        <v>627</v>
+        <v>651</v>
       </c>
     </row>
     <row r="41" spans="1:2" customHeight="1" ht="22.05">
       <c r="B41" s="2" t="s">
-        <v>502</v>
+        <v>519</v>
       </c>
     </row>
     <row r="42" spans="1:2" customHeight="1" ht="22.05">
       <c r="B42" s="2" t="s">
-        <v>628</v>
+        <v>652</v>
       </c>
     </row>
     <row r="43" spans="1:2" customHeight="1" ht="22.05">
@@ -9622,42 +10558,42 @@
     </row>
     <row r="44" spans="1:2" customHeight="1" ht="22.05">
       <c r="B44" s="2" t="s">
-        <v>629</v>
+        <v>653</v>
       </c>
     </row>
     <row r="45" spans="1:2" customHeight="1" ht="22.05">
       <c r="B45" s="2" t="s">
-        <v>630</v>
+        <v>654</v>
       </c>
     </row>
     <row r="46" spans="1:2" customHeight="1" ht="22.05">
       <c r="B46" s="2" t="s">
-        <v>631</v>
+        <v>655</v>
       </c>
     </row>
     <row r="47" spans="1:2" customHeight="1" ht="22.05">
       <c r="B47" s="2" t="s">
-        <v>632</v>
+        <v>656</v>
       </c>
     </row>
     <row r="48" spans="1:2" customHeight="1" ht="22.05">
       <c r="B48" s="2" t="s">
-        <v>633</v>
+        <v>657</v>
       </c>
     </row>
     <row r="49" spans="1:2" customHeight="1" ht="22.05">
       <c r="B49" s="2" t="s">
-        <v>634</v>
+        <v>658</v>
       </c>
     </row>
     <row r="50" spans="1:2" customHeight="1" ht="22.05">
       <c r="B50" s="2" t="s">
-        <v>635</v>
+        <v>659</v>
       </c>
     </row>
     <row r="51" spans="1:2" customHeight="1" ht="22.05">
       <c r="B51" s="2" t="s">
-        <v>636</v>
+        <v>660</v>
       </c>
     </row>
     <row r="52" spans="1:2" customHeight="1" ht="22.05">
@@ -9667,12 +10603,12 @@
     </row>
     <row r="53" spans="1:2" customHeight="1" ht="22.05">
       <c r="B53" s="2" t="s">
-        <v>637</v>
+        <v>661</v>
       </c>
     </row>
     <row r="54" spans="1:2" customHeight="1" ht="22.05">
       <c r="B54" s="2" t="s">
-        <v>638</v>
+        <v>662</v>
       </c>
     </row>
     <row r="55" spans="1:2" customHeight="1" ht="22.05">
@@ -9682,12 +10618,12 @@
     </row>
     <row r="56" spans="1:2" customHeight="1" ht="22.05">
       <c r="B56" s="2" t="s">
-        <v>639</v>
+        <v>663</v>
       </c>
     </row>
     <row r="57" spans="1:2" customHeight="1" ht="22.05">
       <c r="B57" s="2" t="s">
-        <v>640</v>
+        <v>664</v>
       </c>
     </row>
     <row r="58" spans="1:2" customHeight="1" ht="22.05">
@@ -9697,17 +10633,17 @@
     </row>
     <row r="59" spans="1:2" customHeight="1" ht="22.05">
       <c r="B59" s="2" t="s">
-        <v>641</v>
+        <v>665</v>
       </c>
     </row>
     <row r="60" spans="1:2" customHeight="1" ht="22.05">
       <c r="B60" s="2" t="s">
-        <v>642</v>
+        <v>666</v>
       </c>
     </row>
     <row r="61" spans="1:2" customHeight="1" ht="22.05">
       <c r="B61" s="2" t="s">
-        <v>643</v>
+        <v>667</v>
       </c>
     </row>
     <row r="62" spans="1:2" customHeight="1" ht="22.05">
@@ -9717,17 +10653,17 @@
     </row>
     <row r="63" spans="1:2" customHeight="1" ht="22.05">
       <c r="B63" s="2" t="s">
-        <v>644</v>
+        <v>668</v>
       </c>
     </row>
     <row r="64" spans="1:2" customHeight="1" ht="22.05">
       <c r="B64" s="2" t="s">
-        <v>645</v>
+        <v>669</v>
       </c>
     </row>
     <row r="65" spans="1:2" customHeight="1" ht="22.05">
       <c r="B65" s="2" t="s">
-        <v>646</v>
+        <v>670</v>
       </c>
     </row>
     <row r="66" spans="1:2" customHeight="1" ht="22.05">
@@ -9737,37 +10673,37 @@
     </row>
     <row r="67" spans="1:2" customHeight="1" ht="22.05">
       <c r="B67" s="2" t="s">
-        <v>647</v>
+        <v>671</v>
       </c>
     </row>
     <row r="68" spans="1:2" customHeight="1" ht="22.05">
       <c r="B68" s="2" t="s">
-        <v>648</v>
+        <v>672</v>
       </c>
     </row>
     <row r="69" spans="1:2" customHeight="1" ht="22.05">
       <c r="B69" s="2" t="s">
-        <v>649</v>
+        <v>673</v>
       </c>
     </row>
     <row r="70" spans="1:2" customHeight="1" ht="22.05">
       <c r="B70" s="2" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
     </row>
     <row r="71" spans="1:2" customHeight="1" ht="22.05">
       <c r="B71" s="2" t="s">
-        <v>650</v>
+        <v>674</v>
       </c>
     </row>
     <row r="72" spans="1:2" customHeight="1" ht="22.05">
       <c r="B72" s="2" t="s">
-        <v>651</v>
+        <v>675</v>
       </c>
     </row>
     <row r="73" spans="1:2" customHeight="1" ht="22.05">
       <c r="B73" s="2" t="s">
-        <v>652</v>
+        <v>676</v>
       </c>
     </row>
     <row r="74" spans="1:2" customHeight="1" ht="22.05">
@@ -9777,32 +10713,32 @@
     </row>
     <row r="75" spans="1:2" customHeight="1" ht="22.05">
       <c r="B75" s="2" t="s">
-        <v>653</v>
+        <v>677</v>
       </c>
     </row>
     <row r="76" spans="1:2" customHeight="1" ht="22.05">
       <c r="B76" s="2" t="s">
-        <v>654</v>
+        <v>678</v>
       </c>
     </row>
     <row r="77" spans="1:2" customHeight="1" ht="22.05">
       <c r="B77" s="2" t="s">
-        <v>655</v>
+        <v>679</v>
       </c>
     </row>
     <row r="78" spans="1:2" customHeight="1" ht="22.05">
       <c r="B78" s="2" t="s">
-        <v>656</v>
+        <v>680</v>
       </c>
     </row>
     <row r="79" spans="1:2" customHeight="1" ht="22.05">
       <c r="B79" s="2" t="s">
-        <v>657</v>
+        <v>681</v>
       </c>
     </row>
     <row r="80" spans="1:2" customHeight="1" ht="22.05">
       <c r="B80" s="2" t="s">
-        <v>658</v>
+        <v>682</v>
       </c>
     </row>
     <row r="81" spans="1:2" customHeight="1" ht="22.05">
@@ -9812,42 +10748,42 @@
     </row>
     <row r="82" spans="1:2" customHeight="1" ht="22.05">
       <c r="B82" s="2" t="s">
-        <v>659</v>
+        <v>683</v>
       </c>
     </row>
     <row r="83" spans="1:2" customHeight="1" ht="22.05">
       <c r="B83" s="2" t="s">
-        <v>660</v>
+        <v>684</v>
       </c>
     </row>
     <row r="84" spans="1:2" customHeight="1" ht="22.05">
       <c r="B84" s="2" t="s">
-        <v>533</v>
+        <v>556</v>
       </c>
     </row>
     <row r="85" spans="1:2" customHeight="1" ht="22.05">
       <c r="B85" s="2" t="s">
-        <v>661</v>
+        <v>685</v>
       </c>
     </row>
     <row r="86" spans="1:2" customHeight="1" ht="22.05">
       <c r="B86" s="2" t="s">
-        <v>662</v>
+        <v>686</v>
       </c>
     </row>
     <row r="87" spans="1:2" customHeight="1" ht="22.05">
       <c r="B87" s="2" t="s">
-        <v>663</v>
+        <v>687</v>
       </c>
     </row>
     <row r="88" spans="1:2" customHeight="1" ht="22.05">
       <c r="B88" s="2" t="s">
-        <v>664</v>
+        <v>688</v>
       </c>
     </row>
     <row r="89" spans="1:2" customHeight="1" ht="22.05">
       <c r="B89" s="2" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
     </row>
     <row r="90" spans="1:2" customHeight="1" ht="22.05">
@@ -9857,7 +10793,7 @@
     </row>
     <row r="91" spans="1:2" customHeight="1" ht="22.05">
       <c r="B91" s="2" t="s">
-        <v>665</v>
+        <v>689</v>
       </c>
     </row>
     <row r="92" spans="1:2" customHeight="1" ht="22.05">
@@ -9867,17 +10803,17 @@
     </row>
     <row r="93" spans="1:2" customHeight="1" ht="22.05">
       <c r="B93" s="2" t="s">
-        <v>666</v>
+        <v>690</v>
       </c>
     </row>
     <row r="94" spans="1:2" customHeight="1" ht="22.05">
       <c r="B94" s="2" t="s">
-        <v>667</v>
+        <v>691</v>
       </c>
     </row>
     <row r="95" spans="1:2" customHeight="1" ht="22.05">
       <c r="B95" s="2" t="s">
-        <v>668</v>
+        <v>692</v>
       </c>
     </row>
     <row r="96" spans="1:2" customHeight="1" ht="22.05">
@@ -9887,12 +10823,12 @@
     </row>
     <row r="97" spans="1:2" customHeight="1" ht="22.05">
       <c r="B97" s="2" t="s">
-        <v>669</v>
+        <v>693</v>
       </c>
     </row>
     <row r="98" spans="1:2" customHeight="1" ht="22.05">
       <c r="B98" s="2" t="s">
-        <v>670</v>
+        <v>694</v>
       </c>
     </row>
     <row r="99" spans="1:2" customHeight="1" ht="22.05">
@@ -9902,47 +10838,47 @@
     </row>
     <row r="100" spans="1:2" customHeight="1" ht="22.05">
       <c r="B100" s="2" t="s">
-        <v>671</v>
+        <v>695</v>
       </c>
     </row>
     <row r="101" spans="1:2" customHeight="1" ht="22.05">
       <c r="B101" s="2" t="s">
-        <v>672</v>
+        <v>696</v>
       </c>
     </row>
     <row r="102" spans="1:2" customHeight="1" ht="22.05">
       <c r="B102" s="2" t="s">
-        <v>673</v>
+        <v>697</v>
       </c>
     </row>
     <row r="103" spans="1:2" customHeight="1" ht="22.05">
       <c r="B103" s="2" t="s">
-        <v>674</v>
+        <v>698</v>
       </c>
     </row>
     <row r="104" spans="1:2" customHeight="1" ht="22.05">
       <c r="B104" s="2" t="s">
-        <v>675</v>
+        <v>699</v>
       </c>
     </row>
     <row r="105" spans="1:2" customHeight="1" ht="22.05">
       <c r="B105" s="2" t="s">
-        <v>676</v>
+        <v>700</v>
       </c>
     </row>
     <row r="106" spans="1:2" customHeight="1" ht="22.05">
       <c r="B106" s="2" t="s">
-        <v>677</v>
+        <v>701</v>
       </c>
     </row>
     <row r="107" spans="1:2" customHeight="1" ht="22.05">
       <c r="B107" s="2" t="s">
-        <v>678</v>
+        <v>702</v>
       </c>
     </row>
     <row r="108" spans="1:2" customHeight="1" ht="22.05">
       <c r="B108" s="2" t="s">
-        <v>679</v>
+        <v>703</v>
       </c>
     </row>
     <row r="109" spans="1:2" customHeight="1" ht="22.05">
@@ -9952,37 +10888,37 @@
     </row>
     <row r="110" spans="1:2" customHeight="1" ht="22.05">
       <c r="B110" s="2" t="s">
-        <v>680</v>
+        <v>704</v>
       </c>
     </row>
     <row r="111" spans="1:2" customHeight="1" ht="22.05">
       <c r="B111" s="2" t="s">
-        <v>681</v>
+        <v>705</v>
       </c>
     </row>
     <row r="112" spans="1:2" customHeight="1" ht="22.05">
       <c r="B112" s="2" t="s">
-        <v>682</v>
+        <v>706</v>
       </c>
     </row>
     <row r="113" spans="1:2" customHeight="1" ht="22.05">
       <c r="B113" s="2" t="s">
-        <v>683</v>
+        <v>707</v>
       </c>
     </row>
     <row r="114" spans="1:2" customHeight="1" ht="22.05">
       <c r="B114" s="2" t="s">
-        <v>684</v>
+        <v>708</v>
       </c>
     </row>
     <row r="115" spans="1:2" customHeight="1" ht="22.05">
       <c r="B115" s="2" t="s">
-        <v>496</v>
+        <v>512</v>
       </c>
     </row>
     <row r="116" spans="1:2" customHeight="1" ht="22.05">
       <c r="B116" s="2" t="s">
-        <v>685</v>
+        <v>709</v>
       </c>
     </row>
     <row r="117" spans="1:2" customHeight="1" ht="22.05">
@@ -9992,27 +10928,27 @@
     </row>
     <row r="118" spans="1:2" customHeight="1" ht="22.05">
       <c r="B118" s="2" t="s">
-        <v>686</v>
+        <v>710</v>
       </c>
     </row>
     <row r="119" spans="1:2" customHeight="1" ht="22.05">
       <c r="B119" s="2" t="s">
-        <v>687</v>
+        <v>711</v>
       </c>
     </row>
     <row r="120" spans="1:2" customHeight="1" ht="22.05">
       <c r="B120" s="2" t="s">
-        <v>688</v>
+        <v>712</v>
       </c>
     </row>
     <row r="121" spans="1:2" customHeight="1" ht="22.05">
       <c r="B121" s="2" t="s">
-        <v>689</v>
+        <v>713</v>
       </c>
     </row>
     <row r="122" spans="1:2" customHeight="1" ht="22.05">
       <c r="B122" s="2" t="s">
-        <v>690</v>
+        <v>714</v>
       </c>
     </row>
     <row r="123" spans="1:2" customHeight="1" ht="22.05">
@@ -10027,27 +10963,27 @@
     </row>
     <row r="125" spans="1:2" customHeight="1" ht="22.05">
       <c r="B125" s="2" t="s">
-        <v>691</v>
+        <v>715</v>
       </c>
     </row>
     <row r="126" spans="1:2" customHeight="1" ht="22.05">
       <c r="B126" s="2" t="s">
-        <v>692</v>
+        <v>716</v>
       </c>
     </row>
     <row r="127" spans="1:2" customHeight="1" ht="22.05">
       <c r="B127" s="2" t="s">
-        <v>693</v>
+        <v>717</v>
       </c>
     </row>
     <row r="128" spans="1:2" customHeight="1" ht="22.05">
       <c r="B128" s="2" t="s">
-        <v>694</v>
+        <v>718</v>
       </c>
     </row>
     <row r="129" spans="1:2" customHeight="1" ht="22.05">
       <c r="B129" s="2" t="s">
-        <v>695</v>
+        <v>719</v>
       </c>
     </row>
     <row r="130" spans="1:2" customHeight="1" ht="22.05">

</xml_diff>